<commit_message>
Update GEMINI logic code
</commit_message>
<xml_diff>
--- a/data/May/Data_May.xlsx
+++ b/data/May/Data_May.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\May\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8499EE5E-5161-4C66-88F9-A2696A91346E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C407264-DD13-4CF3-9CE2-CE8072A9A7D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01-05" sheetId="4" r:id="rId1"/>
@@ -26,6 +26,7 @@
     <sheet name="14-05" sheetId="15" r:id="rId11"/>
     <sheet name="15-05" sheetId="16" r:id="rId12"/>
     <sheet name="16-05" sheetId="17" r:id="rId13"/>
+    <sheet name="18-05" sheetId="18" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4223" uniqueCount="1403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4558" uniqueCount="1496">
   <si>
     <t>THU 6</t>
   </si>
@@ -4007,36 +4008,54 @@
     <t>AT 16-05</t>
   </si>
   <si>
+    <t>kh ck shop 4210k</t>
+  </si>
+  <si>
     <t>HD021355</t>
   </si>
   <si>
     <t>HD021442</t>
   </si>
   <si>
+    <t>42, đường 21,Khu dân cư bình chiểu, P tam bình (chợ đầu mối nông sản thủ đức)</t>
+  </si>
+  <si>
     <t>Phạm T. Thảo</t>
   </si>
   <si>
     <t>HD021288</t>
   </si>
   <si>
+    <t>63 dương bá trạc p. rạch ông</t>
+  </si>
+  <si>
     <t>VERISKA (YAYANG) - ROOM 104.</t>
   </si>
   <si>
     <t>HD021409</t>
   </si>
   <si>
+    <t>Saigon Europe Hotel, Số 207 đường Đề Thám, phường bến Thành</t>
+  </si>
+  <si>
     <t>chị Huyền</t>
   </si>
   <si>
     <t>HĐ021386</t>
   </si>
   <si>
+    <t>9B nguyễn xí, phường 26</t>
+  </si>
+  <si>
     <t>Nhận hành giúp chị phương (ở Úc) fb Phương My</t>
   </si>
   <si>
     <t>HD021421</t>
   </si>
   <si>
+    <t>126/5h song hành, tân hiệp</t>
+  </si>
+  <si>
     <t>hoc mon</t>
   </si>
   <si>
@@ -4055,21 +4074,45 @@
     <t>HD021213</t>
   </si>
   <si>
+    <t>67 mai chí thọ phường an phú</t>
+  </si>
+  <si>
     <t>Trần Bảo Hân (inst tienbaohen17)</t>
   </si>
   <si>
     <t>HD021310</t>
   </si>
   <si>
+    <t>E4/25a đường Nguyễn Hữu Trí, khu phố 12, thị trấn Tân Túc</t>
+  </si>
+  <si>
     <t>Hiệp fb Đặng Tổ Trinh</t>
   </si>
   <si>
+    <t>HD021271</t>
+  </si>
+  <si>
+    <t>Số 3 hoàng minh giám phường đức nhuận</t>
+  </si>
+  <si>
+    <t>Loan Trần</t>
+  </si>
+  <si>
     <t>HD021379</t>
   </si>
   <si>
+    <t>64/24C hoà bình phường hòa bình</t>
+  </si>
+  <si>
+    <t>Linh Tiêu</t>
+  </si>
+  <si>
     <t>HD021267</t>
   </si>
   <si>
+    <t>97 Ký Con, p. Nguyễn Thái Bình</t>
+  </si>
+  <si>
     <t>HD021227</t>
   </si>
   <si>
@@ -4103,63 +4146,99 @@
     <t>HD021425</t>
   </si>
   <si>
+    <t>287/1/5 thành công, tân thành</t>
+  </si>
+  <si>
+    <t>Ngọc Mỹ Kim</t>
+  </si>
+  <si>
+    <t>HD021327</t>
+  </si>
+  <si>
+    <t>Chung cu topaz elite drgon 2c p4 ta quang buu</t>
+  </si>
+  <si>
+    <t>kh ck shop 1820k</t>
+  </si>
+  <si>
+    <t>Trần Bảo Hân (inst tranbaohan17)</t>
+  </si>
+  <si>
+    <t>HD021309</t>
+  </si>
+  <si>
+    <t>Cẩm Cẩm</t>
+  </si>
+  <si>
+    <t>HD021193</t>
+  </si>
+  <si>
+    <t>150 Hoàng Trọng Mậu Tân Hưng</t>
+  </si>
+  <si>
+    <t>Sam Sam</t>
+  </si>
+  <si>
+    <t>HD021214</t>
+  </si>
+  <si>
+    <t>Sunrise city view tòa B .33 Nguyễn Hữu Thọ phường tân hưng</t>
+  </si>
+  <si>
+    <t>Ann Ann</t>
+  </si>
+  <si>
+    <t>HD021246</t>
+  </si>
+  <si>
+    <t>172 lê thị bạch cát p11</t>
+  </si>
+  <si>
+    <t>HD021369</t>
+  </si>
+  <si>
+    <t>87/10 trần quang cơ phú thạnh</t>
+  </si>
+  <si>
+    <t>HD021282</t>
+  </si>
+  <si>
     <t>287/1/5 thành công, tấn thành</t>
   </si>
   <si>
-    <t>Ngọc Mỹ Kim</t>
-  </si>
-  <si>
-    <t>HD021327</t>
-  </si>
-  <si>
-    <t>Chung cu topaz elite drgon 2c p4 ta quang buu</t>
-  </si>
-  <si>
-    <t>Trần Bảo Hân (inst tranbaohan17)</t>
-  </si>
-  <si>
-    <t>HD021309</t>
-  </si>
-  <si>
-    <t>HD021193</t>
-  </si>
-  <si>
-    <t>Sam Sam</t>
-  </si>
-  <si>
-    <t>HD021214</t>
-  </si>
-  <si>
-    <t>172 lê thị bạch cát p11</t>
-  </si>
-  <si>
-    <t>HD021369</t>
-  </si>
-  <si>
-    <t>87/10 trần quang cơ phú thạnh</t>
-  </si>
-  <si>
-    <t>HD021282</t>
-  </si>
-  <si>
     <t>Thien Phu Nguyen</t>
   </si>
   <si>
     <t>HD021468</t>
   </si>
   <si>
+    <t>Block B - Chung cư RiverGate Residence 151-155 Bến Vân Đồn, Phường Khánh Hội</t>
+  </si>
+  <si>
     <t>Ánh Hoàng</t>
   </si>
   <si>
     <t>HD021275</t>
   </si>
   <si>
+    <t>Stown Tham Lương sảnh B Phường Tân Thới Nhất</t>
+  </si>
+  <si>
     <t>HD021185</t>
   </si>
   <si>
+    <t>Số 207 đường Đề Thám, phường bến Thành</t>
+  </si>
+  <si>
     <t>Mai Sương</t>
   </si>
   <si>
+    <t>HD021469</t>
+  </si>
+  <si>
+    <t>55/3 trần đình xu, phường cầu kho</t>
+  </si>
+  <si>
     <t>Huỳnh Phương Mỹ Duyên</t>
   </si>
   <si>
@@ -4172,91 +4251,292 @@
     <t>Hồng Thắm</t>
   </si>
   <si>
+    <t>27 đông hưng thuận 45 tân hưng thuận</t>
+  </si>
+  <si>
     <t>Heng Stella</t>
   </si>
   <si>
     <t>tân sơn p12</t>
   </si>
   <si>
-    <t>9B nguyễn xí, phường 26</t>
-  </si>
-  <si>
-    <t>Stown Tham Lương sảnh B Phường Tân Thới Nhất</t>
-  </si>
-  <si>
-    <t>42, đường 21,Khu dân cư bình chiểu, P tam bình (chợ đầu mối nông sản thủ đức)</t>
-  </si>
-  <si>
-    <t>67 mai chí thọ phường an phú</t>
-  </si>
-  <si>
-    <t>27 đông hưng thuận 45 tân hưng thuận</t>
-  </si>
-  <si>
-    <t>Linh Tiêu</t>
-  </si>
-  <si>
-    <t>97 Ký Con, p. Nguyễn Thái Bình</t>
-  </si>
-  <si>
-    <t>Block B - Chung cư RiverGate Residence 151-155 Bến Vân Đồn, Phường Khánh Hội</t>
-  </si>
-  <si>
-    <t>HD021271</t>
-  </si>
-  <si>
-    <t>Số 3 hoàng minh giám phường đức nhuận</t>
-  </si>
-  <si>
-    <t>HD021246</t>
-  </si>
-  <si>
-    <t>HD021469</t>
-  </si>
-  <si>
-    <t>55/3 trần đình xu, phường cầu kho</t>
-  </si>
-  <si>
-    <t>Số 207 đường Đề Thám, phường bến Thành</t>
-  </si>
-  <si>
-    <t>Saigon Europe Hotel, Số 207 đường Đề Thám, phường bến Thành</t>
-  </si>
-  <si>
-    <t>Ann Ann</t>
-  </si>
-  <si>
-    <t>Loan Trần</t>
-  </si>
-  <si>
-    <t>64/24C hoà bình phường hòa bình</t>
-  </si>
-  <si>
-    <t>Cẩm Cẩm</t>
-  </si>
-  <si>
-    <t>150 Hoàng Trọng Mậu Tân Hưng</t>
-  </si>
-  <si>
-    <t>Sunrise city view tòa B .33 Nguyễn Hữu Thọ phường tân hưng</t>
-  </si>
-  <si>
-    <t>126/5h song hành, tân hiệp</t>
-  </si>
-  <si>
-    <t>63 dương bá trạc p. rạch ông</t>
-  </si>
-  <si>
-    <t>287/1/5 thành công, tân thành</t>
-  </si>
-  <si>
-    <t>kh ck shop 4210k</t>
-  </si>
-  <si>
-    <t>E4/25a đường Nguyễn Hữu Trí, khu phố 12, thị trấn Tân Túc</t>
-  </si>
-  <si>
-    <t>kh ck shop 1820k</t>
+    <t>NGAY 18-5</t>
+  </si>
+  <si>
+    <t>18-05-2026</t>
+  </si>
+  <si>
+    <t>NIKI</t>
+  </si>
+  <si>
+    <t>AT 18-05</t>
+  </si>
+  <si>
+    <t>Heng Roza (EV38382)</t>
+  </si>
+  <si>
+    <t>Gia Huy nhận của ELIS NGUYỄN ( singapore)</t>
+  </si>
+  <si>
+    <t>HD021334</t>
+  </si>
+  <si>
+    <t>HD021855</t>
+  </si>
+  <si>
+    <t>Quỳnh Nga</t>
+  </si>
+  <si>
+    <t>HD021747</t>
+  </si>
+  <si>
+    <t>Ngọc - fb Naila Unner</t>
+  </si>
+  <si>
+    <t>HD021827</t>
+  </si>
+  <si>
+    <t>Rivergate</t>
+  </si>
+  <si>
+    <t>HD021876</t>
+  </si>
+  <si>
+    <t>Ngọc Hồng Thương</t>
+  </si>
+  <si>
+    <t>HD021553</t>
+  </si>
+  <si>
+    <t>51 đường 81 tân quy</t>
+  </si>
+  <si>
+    <t>PIMVIPA 3883</t>
+  </si>
+  <si>
+    <t>HD021837</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Mỹ Phúc</t>
+  </si>
+  <si>
+    <t>HD021574</t>
+  </si>
+  <si>
+    <t>nha The Sun Avenue (tòa S5) 28 Mai Chí Thọ, An Phú</t>
+  </si>
+  <si>
+    <t>HD021424</t>
+  </si>
+  <si>
+    <t>Gia Tuệ</t>
+  </si>
+  <si>
+    <t>HD021808</t>
+  </si>
+  <si>
+    <t>42/32 trần đại nghĩa, tân tạo a</t>
+  </si>
+  <si>
+    <t>Ngọc</t>
+  </si>
+  <si>
+    <t>HD021842</t>
+  </si>
+  <si>
+    <t>Hoàng Trâm Anh</t>
+  </si>
+  <si>
+    <t>HD021810</t>
+  </si>
+  <si>
+    <t>HSM RIDA CHUON</t>
+  </si>
+  <si>
+    <t>HD021615</t>
+  </si>
+  <si>
+    <t>177c đường số 1 bình hưng hòa b</t>
+  </si>
+  <si>
+    <t>Trúc Nguyễn</t>
+  </si>
+  <si>
+    <t>HD021871</t>
+  </si>
+  <si>
+    <t>38 Đường 6 Linh Chiếu</t>
+  </si>
+  <si>
+    <t>Hợp Vũ</t>
+  </si>
+  <si>
+    <t>HD021640</t>
+  </si>
+  <si>
+    <t>2A Phan Chu Trinh, P Hiệp Phú</t>
+  </si>
+  <si>
+    <t>HD021866</t>
+  </si>
+  <si>
+    <t>Đối diện 110/42 đường số 5 phường 17</t>
+  </si>
+  <si>
+    <t>HD021418</t>
+  </si>
+  <si>
+    <t>Ái Nương</t>
+  </si>
+  <si>
+    <t>HD021666</t>
+  </si>
+  <si>
+    <t>154/33 au dương lân phường 3</t>
+  </si>
+  <si>
+    <t>Trân Nguyễn</t>
+  </si>
+  <si>
+    <t>HD021600</t>
+  </si>
+  <si>
+    <t>HD021539</t>
+  </si>
+  <si>
+    <t>MC Phương Nhi</t>
+  </si>
+  <si>
+    <t>HD021829</t>
+  </si>
+  <si>
+    <t>99 Trần Bá Giao An Nhơn</t>
+  </si>
+  <si>
+    <t>chị Bích Huyền</t>
+  </si>
+  <si>
+    <t>HD021868</t>
+  </si>
+  <si>
+    <t>Số 4 đường số 22 kdc bình hưng</t>
+  </si>
+  <si>
+    <t>HD021775</t>
+  </si>
+  <si>
+    <t>Ngân Ngân</t>
+  </si>
+  <si>
+    <t>Phuong Nguyen</t>
+  </si>
+  <si>
+    <t>HD021530</t>
+  </si>
+  <si>
+    <t>Eco green toà I, HR30710, 39 Nguyễn Văn linh</t>
+  </si>
+  <si>
+    <t>HD021612</t>
+  </si>
+  <si>
+    <t>497/73/5 phan văn trị Phường 5</t>
+  </si>
+  <si>
+    <t>Ngann Lee</t>
+  </si>
+  <si>
+    <t>HD021534</t>
+  </si>
+  <si>
+    <t>222 pasteur, phường xuân hòa</t>
+  </si>
+  <si>
+    <t>2/11 Đường Thiên Phước, Phường 9</t>
+  </si>
+  <si>
+    <t>29/7 Yên Thế, Phường 2</t>
+  </si>
+  <si>
+    <t>Hong Nho + NGUYỄN THỊ DIỄM CHI</t>
+  </si>
+  <si>
+    <t>SU ANH</t>
+  </si>
+  <si>
+    <t>177 Nguyễn Đình Chiểu, p. Xuân Hòa</t>
+  </si>
+  <si>
+    <t>Thinh HB</t>
+  </si>
+  <si>
+    <t>HD021608</t>
+  </si>
+  <si>
+    <t>17 cô giang, phường cầu ông lãnh</t>
+  </si>
+  <si>
+    <t>Tô Tô</t>
+  </si>
+  <si>
+    <t>HD021603</t>
+  </si>
+  <si>
+    <t>46 Lê Thị Riêng, phường Bến Thành</t>
+  </si>
+  <si>
+    <t>56/7 đường Tân Hoà 2 phường Hiệp Phú</t>
+  </si>
+  <si>
+    <t>Vân Thuỳ</t>
+  </si>
+  <si>
+    <t>như fb Đặng Tố Trinh</t>
+  </si>
+  <si>
+    <t>129/34 Nguyễn Văn Công, P. 3</t>
+  </si>
+  <si>
+    <t>11 Nguyễn Bá Huân phường thảo điền</t>
+  </si>
+  <si>
+    <t>HD021620</t>
+  </si>
+  <si>
+    <t>74B/148 thống nhất p15</t>
+  </si>
+  <si>
+    <t>Nguyễn Thảo Uyên</t>
+  </si>
+  <si>
+    <t>HD021746</t>
+  </si>
+  <si>
+    <t>15/32/56 võ duy ninh p22</t>
+  </si>
+  <si>
+    <t>Nga Còi</t>
+  </si>
+  <si>
+    <t>Sửa xe Anh Sơn, liên ấp 2,3,4 Vĩnh Lộc A</t>
+  </si>
+  <si>
+    <t>Central premium lock A</t>
+  </si>
+  <si>
+    <t>Chị Bích Huyền</t>
+  </si>
+  <si>
+    <t>số 4 đường số 22 kdc bình hưng</t>
+  </si>
+  <si>
+    <t>HD021621</t>
+  </si>
+  <si>
+    <t>360 lạc long quân phường 5 (phường hòa bình)</t>
+  </si>
+  <si>
+    <t>HD020691</t>
   </si>
 </sst>
 </file>
@@ -10531,10 +10811,12 @@
   <dimension ref="A1:Q41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
     <col min="3" max="3" width="45" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="93.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
     <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -10673,7 +10955,7 @@
         <v>1314</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>1400</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="5" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -10684,7 +10966,7 @@
         <v>854</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>242</v>
@@ -10720,10 +11002,10 @@
         <v>856</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>1378</v>
+        <v>1322</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>77</v>
@@ -10753,13 +11035,13 @@
         <v>18</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>1321</v>
+        <v>1323</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>1322</v>
+        <v>1324</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>1398</v>
+        <v>1325</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>41</v>
@@ -10789,13 +11071,13 @@
         <v>18</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>1323</v>
+        <v>1326</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>1324</v>
+        <v>1327</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>1390</v>
+        <v>1328</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>63</v>
@@ -10828,13 +11110,13 @@
         <v>18</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>1325</v>
+        <v>1329</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>1326</v>
+        <v>1330</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>1376</v>
+        <v>1331</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>81</v>
@@ -10864,16 +11146,16 @@
         <v>18</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>1327</v>
+        <v>1332</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>1328</v>
+        <v>1333</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>1397</v>
+        <v>1334</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>1329</v>
+        <v>1335</v>
       </c>
       <c r="G10" s="8">
         <v>865</v>
@@ -10900,13 +11182,13 @@
         <v>18</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>1330</v>
+        <v>1336</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>1331</v>
+        <v>1337</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>1332</v>
+        <v>1338</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>77</v>
@@ -10936,13 +11218,13 @@
         <v>18</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>1333</v>
+        <v>1339</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>1334</v>
+        <v>1340</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>1379</v>
+        <v>1341</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>48</v>
@@ -10972,13 +11254,13 @@
         <v>18</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>1335</v>
+        <v>1342</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>1336</v>
+        <v>1343</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>1401</v>
+        <v>1344</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>52</v>
@@ -11011,13 +11293,13 @@
         <v>18</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>1337</v>
+        <v>1345</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>1384</v>
+        <v>1346</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>1385</v>
+        <v>1347</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>355</v>
@@ -11047,13 +11329,13 @@
         <v>18</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>1392</v>
+        <v>1348</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>1338</v>
+        <v>1349</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>1393</v>
+        <v>1350</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>239</v>
@@ -11083,13 +11365,13 @@
         <v>18</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>1381</v>
+        <v>1351</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>1339</v>
+        <v>1352</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>1382</v>
+        <v>1353</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>63</v>
@@ -11122,7 +11404,7 @@
         <v>177</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>1340</v>
+        <v>1354</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>179</v>
@@ -11155,10 +11437,10 @@
         <v>18</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>1341</v>
+        <v>1355</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>1342</v>
+        <v>1356</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>511</v>
@@ -11191,13 +11473,13 @@
         <v>18</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>1343</v>
+        <v>1357</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>1344</v>
+        <v>1358</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>1345</v>
+        <v>1359</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>131</v>
@@ -11227,13 +11509,13 @@
         <v>18</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>1346</v>
+        <v>1360</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>1347</v>
+        <v>1361</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>1348</v>
+        <v>1362</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>77</v>
@@ -11263,13 +11545,13 @@
         <v>18</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>1349</v>
+        <v>1363</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>1350</v>
+        <v>1364</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>1399</v>
+        <v>1365</v>
       </c>
       <c r="F21" s="8" t="s">
         <v>85</v>
@@ -11302,13 +11584,13 @@
         <v>18</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>1352</v>
+        <v>1366</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>1353</v>
+        <v>1367</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>1354</v>
+        <v>1368</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>41</v>
@@ -11333,7 +11615,7 @@
         <v>1314</v>
       </c>
       <c r="M22" s="8" t="s">
-        <v>1402</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="23" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -11341,13 +11623,13 @@
         <v>18</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>1355</v>
+        <v>1370</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>1356</v>
+        <v>1371</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>1401</v>
+        <v>1344</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>52</v>
@@ -11380,13 +11662,13 @@
         <v>18</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>1394</v>
+        <v>1372</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>1357</v>
+        <v>1373</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>1395</v>
+        <v>1374</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>131</v>
@@ -11416,13 +11698,13 @@
         <v>18</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>1358</v>
+        <v>1375</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>1359</v>
+        <v>1376</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>1396</v>
+        <v>1377</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>131</v>
@@ -11452,13 +11734,13 @@
         <v>18</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>1391</v>
+        <v>1378</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>1386</v>
+        <v>1379</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>1360</v>
+        <v>1380</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>239</v>
@@ -11491,10 +11773,10 @@
         <v>748</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>1361</v>
+        <v>1381</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>1362</v>
+        <v>1382</v>
       </c>
       <c r="F27" s="8" t="s">
         <v>85</v>
@@ -11524,13 +11806,13 @@
         <v>18</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>1349</v>
+        <v>1363</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>1363</v>
+        <v>1383</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>1351</v>
+        <v>1384</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>85</v>
@@ -11563,13 +11845,13 @@
         <v>18</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>1364</v>
+        <v>1385</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>1365</v>
+        <v>1386</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
       <c r="F29" s="7" t="s">
         <v>186</v>
@@ -11599,13 +11881,13 @@
         <v>18</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>1366</v>
+        <v>1388</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>1367</v>
+        <v>1389</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>1377</v>
+        <v>1390</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>29</v>
@@ -11635,13 +11917,13 @@
         <v>18</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>1323</v>
+        <v>1326</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>1368</v>
+        <v>1391</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>1389</v>
+        <v>1392</v>
       </c>
       <c r="F31" s="6" t="s">
         <v>63</v>
@@ -11674,13 +11956,13 @@
         <v>18</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>1369</v>
+        <v>1393</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>1387</v>
+        <v>1394</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>1388</v>
+        <v>1395</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>63</v>
@@ -11710,13 +11992,13 @@
         <v>18</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>1370</v>
+        <v>1396</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>1371</v>
+        <v>1397</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>1372</v>
+        <v>1398</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>48</v>
@@ -11785,10 +12067,10 @@
         <v>18</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>1373</v>
+        <v>1399</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>1380</v>
+        <v>1400</v>
       </c>
       <c r="F35" s="4" t="s">
         <v>29</v>
@@ -11821,7 +12103,7 @@
         <v>18</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>1374</v>
+        <v>1401</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>1033</v>
@@ -11896,7 +12178,7 @@
         <v>426</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>1375</v>
+        <v>1402</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>70</v>
@@ -12060,6 +12342,1505 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+  <dimension ref="A1:P41"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="39.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1403</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>1470</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>440</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G3" s="6">
+        <v>0</v>
+      </c>
+      <c r="H3" s="6">
+        <v>30</v>
+      </c>
+      <c r="I3" s="6">
+        <f t="shared" ref="I3" si="0">G3-H3</f>
+        <v>-30</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>1405</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="3">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3">
+        <v>60</v>
+      </c>
+      <c r="I4" s="3">
+        <f>G4-H4</f>
+        <v>-60</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" s="3">
+        <v>30</v>
+      </c>
+      <c r="H5" s="3">
+        <v>30</v>
+      </c>
+      <c r="I5" s="3">
+        <f>G5-H5</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>630</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="G6" s="8">
+        <v>0</v>
+      </c>
+      <c r="H6" s="8">
+        <v>30</v>
+      </c>
+      <c r="I6" s="8">
+        <f>G6-H6</f>
+        <v>-30</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>1469</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>1468</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G7" s="6">
+        <v>30</v>
+      </c>
+      <c r="H7" s="6">
+        <v>30</v>
+      </c>
+      <c r="I7" s="6">
+        <f t="shared" ref="I7:I41" si="1">G7-H7</f>
+        <v>0</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>1399</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>1400</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="3">
+        <v>595</v>
+      </c>
+      <c r="H8" s="3">
+        <v>35</v>
+      </c>
+      <c r="I8" s="3">
+        <f t="shared" ref="I8" si="2">G8-H8</f>
+        <v>560</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>1366</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>1493</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>1368</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="8">
+        <v>380</v>
+      </c>
+      <c r="H9" s="8">
+        <v>30</v>
+      </c>
+      <c r="I9" s="8">
+        <f t="shared" si="1"/>
+        <v>350</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="8" t="s">
+        <v>1404</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>1407</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>1495</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>763</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" s="8">
+        <v>0</v>
+      </c>
+      <c r="H10" s="8">
+        <v>30</v>
+      </c>
+      <c r="I10" s="8">
+        <f t="shared" si="1"/>
+        <v>-30</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="8" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>1408</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>1409</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>1467</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G11" s="6">
+        <v>0</v>
+      </c>
+      <c r="H11" s="6">
+        <v>25</v>
+      </c>
+      <c r="I11" s="6">
+        <f t="shared" si="1"/>
+        <v>-25</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>1078</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>1410</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>1080</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" s="8">
+        <v>0</v>
+      </c>
+      <c r="H12" s="8">
+        <v>30</v>
+      </c>
+      <c r="I12" s="8">
+        <f t="shared" si="1"/>
+        <v>-30</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="8" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>1411</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>1412</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>1478</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="G13" s="5">
+        <v>850</v>
+      </c>
+      <c r="H13" s="5">
+        <v>30</v>
+      </c>
+      <c r="I13" s="5">
+        <f t="shared" si="1"/>
+        <v>820</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="5" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>1413</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>1414</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>1415</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="G14" s="6">
+        <v>1075</v>
+      </c>
+      <c r="H14" s="6">
+        <v>25</v>
+      </c>
+      <c r="I14" s="6">
+        <f t="shared" si="1"/>
+        <v>1050</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>537</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>1416</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G15" s="6">
+        <v>1065</v>
+      </c>
+      <c r="H15" s="6">
+        <v>25</v>
+      </c>
+      <c r="I15" s="6">
+        <f t="shared" si="1"/>
+        <v>1040</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>1417</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>1418</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>1419</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="G16" s="8">
+        <v>0</v>
+      </c>
+      <c r="H16" s="8">
+        <v>30</v>
+      </c>
+      <c r="I16" s="8">
+        <f t="shared" si="1"/>
+        <v>-30</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="8" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>1420</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>1421</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>630</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="G17" s="8">
+        <v>0</v>
+      </c>
+      <c r="H17" s="8">
+        <v>25</v>
+      </c>
+      <c r="I17" s="8">
+        <f t="shared" si="1"/>
+        <v>-25</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K17" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="8" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>1422</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>1423</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>1424</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G18" s="3">
+        <v>890</v>
+      </c>
+      <c r="H18" s="3">
+        <v>30</v>
+      </c>
+      <c r="I18" s="3">
+        <f t="shared" si="1"/>
+        <v>860</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>966</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>1425</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>968</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G19" s="3">
+        <v>380</v>
+      </c>
+      <c r="H19" s="3">
+        <v>30</v>
+      </c>
+      <c r="I19" s="3">
+        <f t="shared" si="1"/>
+        <v>350</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>1426</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>1427</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>1428</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" s="8">
+        <v>0</v>
+      </c>
+      <c r="H20" s="8">
+        <v>30</v>
+      </c>
+      <c r="I20" s="8">
+        <f t="shared" si="1"/>
+        <v>-30</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="8" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>1429</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>1430</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>1466</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G21" s="6">
+        <v>25</v>
+      </c>
+      <c r="H21" s="6">
+        <v>25</v>
+      </c>
+      <c r="I21" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>1404</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>1431</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>1432</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>1482</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G22" s="3">
+        <v>1020</v>
+      </c>
+      <c r="H22" s="3">
+        <v>30</v>
+      </c>
+      <c r="I22" s="3">
+        <f t="shared" si="1"/>
+        <v>990</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>1433</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>1434</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>1435</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G23" s="8">
+        <v>0</v>
+      </c>
+      <c r="H23" s="8">
+        <v>30</v>
+      </c>
+      <c r="I23" s="8">
+        <f t="shared" si="1"/>
+        <v>-30</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="8" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>1436</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>1437</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>1438</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G24" s="3">
+        <v>0</v>
+      </c>
+      <c r="H24" s="3">
+        <v>30</v>
+      </c>
+      <c r="I24" s="3">
+        <f t="shared" si="1"/>
+        <v>-30</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>1488</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>1489</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G25" s="8">
+        <v>0</v>
+      </c>
+      <c r="H25" s="8">
+        <v>35</v>
+      </c>
+      <c r="I25" s="8">
+        <f t="shared" si="1"/>
+        <v>-35</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K25" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="8" t="s">
+        <v>1404</v>
+      </c>
+      <c r="M25" s="8" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>1439</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>1440</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>1441</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="G26" s="5">
+        <v>600</v>
+      </c>
+      <c r="H26" s="5">
+        <v>30</v>
+      </c>
+      <c r="I26" s="5">
+        <f t="shared" si="1"/>
+        <v>570</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="K26" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="5" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>1480</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>1442</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>1443</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G27" s="3">
+        <v>295</v>
+      </c>
+      <c r="H27" s="3">
+        <v>25</v>
+      </c>
+      <c r="I27" s="3">
+        <f t="shared" si="1"/>
+        <v>270</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>1404</v>
+      </c>
+      <c r="M27" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>1473</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>1474</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G28" s="6">
+        <v>915</v>
+      </c>
+      <c r="H28" s="6">
+        <v>25</v>
+      </c>
+      <c r="I28" s="6">
+        <f t="shared" si="1"/>
+        <v>890</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>1485</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>1486</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>1487</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G29" s="3">
+        <v>1190</v>
+      </c>
+      <c r="H29" s="3">
+        <v>20</v>
+      </c>
+      <c r="I29" s="3">
+        <f t="shared" si="1"/>
+        <v>1170</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L29" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>1228</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>1444</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>1490</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G30" s="8">
+        <v>980</v>
+      </c>
+      <c r="H30" s="8">
+        <v>30</v>
+      </c>
+      <c r="I30" s="8">
+        <f t="shared" si="1"/>
+        <v>950</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K30" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L30" s="8" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>1445</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>1446</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>1447</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G31" s="8">
+        <v>380</v>
+      </c>
+      <c r="H31" s="8">
+        <v>30</v>
+      </c>
+      <c r="I31" s="8">
+        <f t="shared" si="1"/>
+        <v>350</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K31" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L31" s="8" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>1448</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>1449</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>1471</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G32" s="6">
+        <v>765</v>
+      </c>
+      <c r="H32" s="6">
+        <v>25</v>
+      </c>
+      <c r="I32" s="6">
+        <f t="shared" si="1"/>
+        <v>740</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L32" s="6" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="33" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>1475</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>1476</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>1477</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G33" s="6">
+        <v>855</v>
+      </c>
+      <c r="H33" s="6">
+        <v>25</v>
+      </c>
+      <c r="I33" s="6">
+        <f t="shared" si="1"/>
+        <v>830</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L33" s="6" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="34" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>1450</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>1481</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G34" s="3">
+        <v>0</v>
+      </c>
+      <c r="H34" s="3">
+        <v>25</v>
+      </c>
+      <c r="I34" s="3">
+        <f t="shared" si="1"/>
+        <v>-25</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L34" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="35" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>1451</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>1452</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>1453</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G35" s="3">
+        <v>885</v>
+      </c>
+      <c r="H35" s="3">
+        <v>25</v>
+      </c>
+      <c r="I35" s="3">
+        <f t="shared" si="1"/>
+        <v>860</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K35" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L35" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="36" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>1455</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>1456</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G36" s="8">
+        <v>695</v>
+      </c>
+      <c r="H36" s="8">
+        <v>35</v>
+      </c>
+      <c r="I36" s="8">
+        <f t="shared" si="1"/>
+        <v>660</v>
+      </c>
+      <c r="J36" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K36" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L36" s="8" t="s">
+        <v>1404</v>
+      </c>
+      <c r="M36" s="8" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="37" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>1491</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>1457</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>1492</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G37" s="8">
+        <v>820</v>
+      </c>
+      <c r="H37" s="8">
+        <v>0</v>
+      </c>
+      <c r="I37" s="8">
+        <f t="shared" si="1"/>
+        <v>820</v>
+      </c>
+      <c r="J37" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K37" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L37" s="8" t="s">
+        <v>1404</v>
+      </c>
+      <c r="M37" s="8" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="38" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>1458</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>1483</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>1484</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G38" s="3">
+        <v>915</v>
+      </c>
+      <c r="H38" s="3">
+        <v>25</v>
+      </c>
+      <c r="I38" s="3">
+        <f t="shared" si="1"/>
+        <v>890</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L38" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="39" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>1460</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>1461</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="G39" s="8">
+        <v>980</v>
+      </c>
+      <c r="H39" s="8">
+        <v>30</v>
+      </c>
+      <c r="I39" s="8">
+        <f t="shared" si="1"/>
+        <v>950</v>
+      </c>
+      <c r="J39" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K39" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L39" s="8" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="40" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>1479</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>1462</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>1463</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G40" s="3">
+        <v>815</v>
+      </c>
+      <c r="H40" s="3">
+        <v>25</v>
+      </c>
+      <c r="I40" s="3">
+        <f t="shared" si="1"/>
+        <v>790</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L40" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="41" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>1464</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>1465</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>1494</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="G41" s="8">
+        <v>985</v>
+      </c>
+      <c r="H41" s="8">
+        <v>25</v>
+      </c>
+      <c r="I41" s="8">
+        <f t="shared" si="1"/>
+        <v>960</v>
+      </c>
+      <c r="J41" s="8" t="s">
+        <v>1406</v>
+      </c>
+      <c r="K41" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L41" s="8" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update 21-05 report and logic
</commit_message>
<xml_diff>
--- a/data/May/Data_May.xlsx
+++ b/data/May/Data_May.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\May\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E3870DF-F153-4CC6-8F1F-23A7C7D4D5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7966C60-AF95-46DC-9E75-2EDAF6FB8348}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01-05" sheetId="4" r:id="rId1"/>
@@ -29,6 +29,7 @@
     <sheet name="18-05" sheetId="18" r:id="rId14"/>
     <sheet name="19-05" sheetId="19" r:id="rId15"/>
     <sheet name="20-05" sheetId="20" r:id="rId16"/>
+    <sheet name="21-05" sheetId="21" r:id="rId17"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5075" uniqueCount="1642">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5425" uniqueCount="1745">
   <si>
     <t>THU 6</t>
   </si>
@@ -4751,21 +4752,33 @@
     <t>NGAY 20-5</t>
   </si>
   <si>
+    <t>20-05-2026</t>
+  </si>
+  <si>
+    <t>Jess-9244</t>
+  </si>
+  <si>
+    <t>275/14B1 Dạng Nguyên Cẩn, Phường Phú Lâm</t>
+  </si>
+  <si>
     <t>AT 20-05</t>
   </si>
   <si>
-    <t>20-05-2026</t>
-  </si>
-  <si>
-    <t>Jess-9244</t>
-  </si>
-  <si>
     <t>VICKY TRẦN</t>
   </si>
   <si>
+    <t>Đắc Hội Express 127/17 bình lợi p13</t>
+  </si>
+  <si>
     <t>hsu_myat to</t>
   </si>
   <si>
+    <t>HD022406</t>
+  </si>
+  <si>
+    <t>2A/14, Nguyễn Thị Minh Khai, P. Đakao</t>
+  </si>
+  <si>
     <t>Bé Hiền - fb Yudy Phạm</t>
   </si>
   <si>
@@ -4796,27 +4809,48 @@
     <t>Vincom đồng khởi, 45 lý tự trọng, căn hộ 2604</t>
   </si>
   <si>
+    <t>HD022255</t>
+  </si>
+  <si>
+    <t>Tòa nhà C22 Building Số G5, Đường C22, Phường 12</t>
+  </si>
+  <si>
     <t>Thanh Yến</t>
   </si>
   <si>
     <t>HD022266</t>
   </si>
   <si>
+    <t>188/4 đường thới an 16 phường thới an</t>
+  </si>
+  <si>
     <t>HƯƠNG</t>
   </si>
   <si>
     <t>HD022382</t>
   </si>
   <si>
+    <t>7g đường số 8 tân hưng</t>
+  </si>
+  <si>
     <t>Vận</t>
   </si>
   <si>
     <t>HD022293</t>
   </si>
   <si>
+    <t>Tháp RS6, chung cư Richstar 2, số 239 Hoà Bình, phường Phú Thạnh</t>
+  </si>
+  <si>
+    <t>nguyen lý</t>
+  </si>
+  <si>
     <t>HD022279</t>
   </si>
   <si>
+    <t>62/7h ấp 3 xã xuaabn thơi thượng</t>
+  </si>
+  <si>
     <t>Ý nhi</t>
   </si>
   <si>
@@ -4853,6 +4887,12 @@
     <t>HD022286</t>
   </si>
   <si>
+    <t>179/13A hoà bình Phường Hiệp Tân</t>
+  </si>
+  <si>
+    <t>Lyly My</t>
+  </si>
+  <si>
     <t>HD022377</t>
   </si>
   <si>
@@ -4868,6 +4908,9 @@
     <t>HD022263</t>
   </si>
   <si>
+    <t>1414 huỳnh tấn phát p phú mỹ</t>
+  </si>
+  <si>
     <t>Huyentran Nguyen</t>
   </si>
   <si>
@@ -4892,9 +4935,18 @@
     <t>HD022412</t>
   </si>
   <si>
+    <t>101 đông hưng thuận42 phường tân hưng thuận</t>
+  </si>
+  <si>
+    <t>ms Linh</t>
+  </si>
+  <si>
     <t>HD022275</t>
   </si>
   <si>
+    <t>141A đường số 1 phường Thông Tây Hội</t>
+  </si>
+  <si>
     <t>HD022267</t>
   </si>
   <si>
@@ -4907,43 +4959,16 @@
     <t>HD022196</t>
   </si>
   <si>
+    <t>181 đường số 79 phường tân quy</t>
+  </si>
+  <si>
     <t>Moon Nguyễn</t>
   </si>
   <si>
     <t>HD022375</t>
   </si>
   <si>
-    <t>ms Linh</t>
-  </si>
-  <si>
-    <t>141A đường số 1 phường Thông Tây Hội</t>
-  </si>
-  <si>
-    <t>Đắc Hội Express 127/17 bình lợi p13</t>
-  </si>
-  <si>
-    <t>275/14B1 Dạng Nguyên Cẩn, Phường Phú Lâm</t>
-  </si>
-  <si>
-    <t>179/13A hoà bình Phường Hiệp Tân</t>
-  </si>
-  <si>
-    <t>Tháp RS6, chung cư Richstar 2, số 239 Hoà Bình, phường Phú Thạnh</t>
-  </si>
-  <si>
-    <t>1414 huỳnh tấn phát p phú mỹ</t>
-  </si>
-  <si>
-    <t>nguyen lý</t>
-  </si>
-  <si>
-    <t>62/7h ấp 3 xã xuaabn thơi thượng</t>
-  </si>
-  <si>
-    <t>101 đông hưng thuận42 phường tân hưng thuận</t>
-  </si>
-  <si>
-    <t>Lyly My</t>
+    <t>16 kim ngân, khu dân cư phong phu 4, xã phong phú</t>
   </si>
   <si>
     <t>Ngoc_Ann tiktok gingeri 16:39</t>
@@ -4955,28 +4980,313 @@
     <t>1/7 nguyễn văn yên tân thới hoà</t>
   </si>
   <si>
-    <t>188/4 đường thới an 16 phường thới an</t>
-  </si>
-  <si>
-    <t>16 kim ngân, khu dân cư phong phu 4, xã phong phú</t>
-  </si>
-  <si>
-    <t>7g đường số 8 tân hưng</t>
-  </si>
-  <si>
-    <t>181 đường số 79 phường tân quy</t>
-  </si>
-  <si>
-    <t>HD022255</t>
-  </si>
-  <si>
-    <t>Tòa nhà C22 Building Số G5, Đường C22, Phường 12</t>
-  </si>
-  <si>
-    <t>HD022406</t>
-  </si>
-  <si>
-    <t>2A/14, Nguyễn Thị Minh Khai, P. Đakao</t>
+    <t>NGAY 21-5</t>
+  </si>
+  <si>
+    <t>AT 21-05</t>
+  </si>
+  <si>
+    <t>21-05-2026</t>
+  </si>
+  <si>
+    <t>Anh Trúc Huỳnh</t>
+  </si>
+  <si>
+    <t>HD022586</t>
+  </si>
+  <si>
+    <t>HD022495</t>
+  </si>
+  <si>
+    <t>BN182 miki chouchou Fb.</t>
+  </si>
+  <si>
+    <t>HD022533</t>
+  </si>
+  <si>
+    <t>Hana Le</t>
+  </si>
+  <si>
+    <t>HD022573</t>
+  </si>
+  <si>
+    <t>Giap Anh Tuyet</t>
+  </si>
+  <si>
+    <t>HD022508</t>
+  </si>
+  <si>
+    <t>Bùi Vĩ Thương</t>
+  </si>
+  <si>
+    <t>HD022636</t>
+  </si>
+  <si>
+    <t>3273 phạm thế hiển, p7</t>
+  </si>
+  <si>
+    <t>HD022429</t>
+  </si>
+  <si>
+    <t>HD022628</t>
+  </si>
+  <si>
+    <t>My Yến</t>
+  </si>
+  <si>
+    <t>HD022525</t>
+  </si>
+  <si>
+    <t>Hải Yến</t>
+  </si>
+  <si>
+    <t>HD003936</t>
+  </si>
+  <si>
+    <t>319/17 lê văn thọ p9</t>
+  </si>
+  <si>
+    <t>Hoang Linh Le</t>
+  </si>
+  <si>
+    <t>HD022460</t>
+  </si>
+  <si>
+    <t>Chị Oanh</t>
+  </si>
+  <si>
+    <t>HD022599</t>
+  </si>
+  <si>
+    <t>291 hùng vương phương an đông</t>
+  </si>
+  <si>
+    <t>HD022451</t>
+  </si>
+  <si>
+    <t>58E cao thắng,p5 (Viện chăm sóc da aperio)</t>
+  </si>
+  <si>
+    <t>Linh Ngô</t>
+  </si>
+  <si>
+    <t>HD022618</t>
+  </si>
+  <si>
+    <t>Lan Phạm</t>
+  </si>
+  <si>
+    <t>HD022621</t>
+  </si>
+  <si>
+    <t>685 âu cơ p tân thành - lô C</t>
+  </si>
+  <si>
+    <t>Sorinna items PhnomPenh ( Meng Kheang customer )</t>
+  </si>
+  <si>
+    <t>HD022445</t>
+  </si>
+  <si>
+    <t>301 phạm ngũ lão</t>
+  </si>
+  <si>
+    <t>01우준</t>
+  </si>
+  <si>
+    <t>HD022601</t>
+  </si>
+  <si>
+    <t>HD022341</t>
+  </si>
+  <si>
+    <t>352/4g lê văn quới, bình hưng hoà A</t>
+  </si>
+  <si>
+    <t>thuy vy</t>
+  </si>
+  <si>
+    <t>HD022620</t>
+  </si>
+  <si>
+    <t>HD022604</t>
+  </si>
+  <si>
+    <t>Mỹ Vinh</t>
+  </si>
+  <si>
+    <t>HD022560</t>
+  </si>
+  <si>
+    <t>HD022503</t>
+  </si>
+  <si>
+    <t>HD022383</t>
+  </si>
+  <si>
+    <t>Nguyễn Yến Nhi</t>
+  </si>
+  <si>
+    <t>HD022491</t>
+  </si>
+  <si>
+    <t>Khánh Thư Nguyen</t>
+  </si>
+  <si>
+    <t>HD022626</t>
+  </si>
+  <si>
+    <t>88 dien Hồng phường 1</t>
+  </si>
+  <si>
+    <t>chủ mau - fb Hana Ngo</t>
+  </si>
+  <si>
+    <t>HD022615</t>
+  </si>
+  <si>
+    <t>Quỳnh Nhi</t>
+  </si>
+  <si>
+    <t>HD022493</t>
+  </si>
+  <si>
+    <t>Mỹ ý</t>
+  </si>
+  <si>
+    <t>HD022613</t>
+  </si>
+  <si>
+    <t>HD022430</t>
+  </si>
+  <si>
+    <t>HD022342</t>
+  </si>
+  <si>
+    <t>NHƯ- Khanh sale- airmy</t>
+  </si>
+  <si>
+    <t>HD022551</t>
+  </si>
+  <si>
+    <t>144C Trần Thị Trọng, Phường 15</t>
+  </si>
+  <si>
+    <t>Nguyễn Thanh Ngân</t>
+  </si>
+  <si>
+    <t>HD022575</t>
+  </si>
+  <si>
+    <t>159c /18a dạ nam, chánh hưng</t>
+  </si>
+  <si>
+    <t>Huỳnh Mẫn</t>
+  </si>
+  <si>
+    <t>HD022522</t>
+  </si>
+  <si>
+    <t>1362 tỉnh lộ 10 tân tạo</t>
+  </si>
+  <si>
+    <t>VVI EVA</t>
+  </si>
+  <si>
+    <t>Toà Aster - Urban green (đối diện Vạn Phúc)</t>
+  </si>
+  <si>
+    <t>163 Đường Trương Thị Hoa, phường Tân Thái Hiệp</t>
+  </si>
+  <si>
+    <t>334/33/1C Chu văn an, phường 12</t>
+  </si>
+  <si>
+    <t>Số 64 dg 38 hiep binh chanh</t>
+  </si>
+  <si>
+    <t>Đảo kim cương phường bình trưng tây</t>
+  </si>
+  <si>
+    <t>PHƯƠNG DUNG</t>
+  </si>
+  <si>
+    <t>23/4A đường 48 khu phố 6 hiệp bình chánh</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Kim Hoàng</t>
+  </si>
+  <si>
+    <t>265 Nơ Trang Long, phường Bình Lợi Trung</t>
+  </si>
+  <si>
+    <t>HD022442</t>
+  </si>
+  <si>
+    <t>314 Điện Biên Phủ, Phường Vườn Lài</t>
+  </si>
+  <si>
+    <t>Aqua1 vinhome bason bến nghé</t>
+  </si>
+  <si>
+    <t>Thuy Thuy</t>
+  </si>
+  <si>
+    <t>141 Hùng Vương phường 4</t>
+  </si>
+  <si>
+    <t>người nhận Hồng Sơn fb Duong Hyun</t>
+  </si>
+  <si>
+    <t>135 Bạch Đằng, phường Tân Sơn Hòa (Phường 2) (CÔNG TY LÊ GIA EXPRESS)</t>
+  </si>
+  <si>
+    <t>320/14 nguyễn văn linh phường bình thuận</t>
+  </si>
+  <si>
+    <t>Lý Thanh Tâm</t>
+  </si>
+  <si>
+    <t>HD022564</t>
+  </si>
+  <si>
+    <t>71/6/16 lê tấn bê an lạc</t>
+  </si>
+  <si>
+    <t>007 Lô B, Đường C6, Chung cư Tây Thạnh</t>
+  </si>
+  <si>
+    <t>90 a lê lăng Phú thọ hoà</t>
+  </si>
+  <si>
+    <t>Tháp v3 Chung cư sun rise city south 23 nguyễn hữu thọ tân hưng</t>
+  </si>
+  <si>
+    <t>67 Trang từ phường 14</t>
+  </si>
+  <si>
+    <t>Phạm Thị Minh Tuyền</t>
+  </si>
+  <si>
+    <t>180/1T QL1A Tân Phú</t>
+  </si>
+  <si>
+    <t>Pé Thỏ</t>
+  </si>
+  <si>
+    <t>1002 tạ quang bửu f6 Chung cư the pegasuite1 (zone1)</t>
+  </si>
+  <si>
+    <t>HD022455</t>
+  </si>
+  <si>
+    <t>427/22 le van quoi binh tri dong A</t>
+  </si>
+  <si>
+    <t>chung cư Ruby - cổng 2, đường Tân Thắng, P. Tân Sơn Nhì</t>
+  </si>
+  <si>
+    <t>HD020811</t>
   </si>
 </sst>
 </file>
@@ -5055,7 +5365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -5071,6 +5381,9 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6599,7 +6912,7 @@
         <v>30</v>
       </c>
       <c r="I35" s="6">
-        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I56" si="1">G35-H35</f>
         <v>30</v>
       </c>
       <c r="J35" s="6" t="s">
@@ -15347,10 +15660,12 @@
   <dimension ref="A1:Q34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
     <col min="3" max="3" width="27.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="60.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
     <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -15450,7 +15765,7 @@
         <v>24</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="4" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -15461,10 +15776,10 @@
         <v>18</v>
       </c>
       <c r="C4" s="8" t="s">
+        <v>1567</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>1568</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>1623</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>127</v>
@@ -15480,13 +15795,13 @@
         <v>-30</v>
       </c>
       <c r="J4" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K4" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="5" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -15522,7 +15837,7 @@
         <v>24</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -15533,10 +15848,10 @@
         <v>18</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>1622</v>
+        <v>1571</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>81</v>
@@ -15558,7 +15873,7 @@
         <v>24</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="7" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -15566,13 +15881,13 @@
         <v>18</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>1570</v>
+        <v>1572</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>1640</v>
+        <v>1573</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>1641</v>
+        <v>1574</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>63</v>
@@ -15594,7 +15909,7 @@
         <v>24</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="8" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -15602,13 +15917,13 @@
         <v>18</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>1571</v>
+        <v>1575</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>1572</v>
+        <v>1576</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>1573</v>
+        <v>1577</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>127</v>
@@ -15624,13 +15939,13 @@
         <v>1850</v>
       </c>
       <c r="J8" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L8" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="9" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -15638,13 +15953,13 @@
         <v>18</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>1574</v>
+        <v>1578</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>1575</v>
+        <v>1579</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>1576</v>
+        <v>1580</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>85</v>
@@ -15660,13 +15975,13 @@
         <v>870</v>
       </c>
       <c r="J9" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L9" s="8" t="s">
-        <v>1567</v>
       </c>
       <c r="M9" s="8" t="s">
         <v>288</v>
@@ -15677,10 +15992,10 @@
         <v>18</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>1577</v>
+        <v>1581</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>1578</v>
+        <v>1582</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>1278</v>
@@ -15699,13 +16014,13 @@
         <v>780</v>
       </c>
       <c r="J10" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K10" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L10" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -15716,10 +16031,10 @@
         <v>777</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>1579</v>
+        <v>1583</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>1580</v>
+        <v>1584</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>63</v>
@@ -15741,7 +16056,7 @@
         <v>24</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="12" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -15752,10 +16067,10 @@
         <v>1058</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>1638</v>
+        <v>1585</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>1639</v>
+        <v>1586</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>102</v>
@@ -15777,7 +16092,7 @@
         <v>24</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="13" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -15785,13 +16100,13 @@
         <v>18</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>1581</v>
+        <v>1587</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>1582</v>
+        <v>1588</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>1634</v>
+        <v>1589</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>29</v>
@@ -15807,13 +16122,13 @@
         <v>820</v>
       </c>
       <c r="J13" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L13" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="14" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -15821,13 +16136,13 @@
         <v>18</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>1583</v>
+        <v>1590</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>1584</v>
+        <v>1591</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>1636</v>
+        <v>1592</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>131</v>
@@ -15843,13 +16158,13 @@
         <v>-30</v>
       </c>
       <c r="J14" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K14" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L14" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="15" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -15857,13 +16172,13 @@
         <v>18</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>1585</v>
+        <v>1593</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>1586</v>
+        <v>1594</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>1625</v>
+        <v>1595</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>85</v>
@@ -15879,13 +16194,13 @@
         <v>350</v>
       </c>
       <c r="J15" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K15" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L15" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="16" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -15893,13 +16208,13 @@
         <v>18</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>1627</v>
+        <v>1596</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>1587</v>
+        <v>1597</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>1628</v>
+        <v>1598</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>1335</v>
@@ -15915,13 +16230,13 @@
         <v>790</v>
       </c>
       <c r="J16" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K16" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L16" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="17" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -15929,13 +16244,13 @@
         <v>18</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>1588</v>
+        <v>1599</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>1589</v>
+        <v>1600</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>1590</v>
+        <v>1601</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>98</v>
@@ -15957,7 +16272,7 @@
         <v>24</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="18" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -15965,13 +16280,13 @@
         <v>18</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>1591</v>
+        <v>1602</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>1592</v>
+        <v>1603</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>1593</v>
+        <v>1604</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>102</v>
@@ -15993,7 +16308,7 @@
         <v>24</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="19" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -16001,10 +16316,10 @@
         <v>18</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>1594</v>
+        <v>1605</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>1595</v>
+        <v>1606</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>1281</v>
@@ -16023,13 +16338,13 @@
         <v>-30</v>
       </c>
       <c r="J19" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K19" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L19" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="20" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -16037,13 +16352,13 @@
         <v>18</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>1596</v>
+        <v>1607</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>1597</v>
+        <v>1608</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>1598</v>
+        <v>1609</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>355</v>
@@ -16065,7 +16380,7 @@
         <v>24</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="21" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -16073,13 +16388,13 @@
         <v>18</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>1574</v>
+        <v>1578</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>1599</v>
+        <v>1610</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>1624</v>
+        <v>1611</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>85</v>
@@ -16095,13 +16410,13 @@
         <v>770</v>
       </c>
       <c r="J21" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K21" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L21" s="8" t="s">
-        <v>1567</v>
       </c>
       <c r="M21" s="8" t="s">
         <v>288</v>
@@ -16112,13 +16427,13 @@
         <v>18</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>1630</v>
+        <v>1612</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>1600</v>
+        <v>1613</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>1601</v>
+        <v>1614</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>29</v>
@@ -16134,13 +16449,13 @@
         <v>1500</v>
       </c>
       <c r="J22" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K22" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L22" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="23" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -16151,7 +16466,7 @@
         <v>558</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>1602</v>
+        <v>1615</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>560</v>
@@ -16176,7 +16491,7 @@
         <v>24</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="24" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -16184,13 +16499,13 @@
         <v>18</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>1603</v>
+        <v>1616</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>1604</v>
+        <v>1617</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>1626</v>
+        <v>1618</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>131</v>
@@ -16206,13 +16521,13 @@
         <v>990</v>
       </c>
       <c r="J24" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K24" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K24" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L24" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="25" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -16220,13 +16535,13 @@
         <v>18</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>1605</v>
+        <v>1619</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>1606</v>
+        <v>1620</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>1607</v>
+        <v>1621</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>63</v>
@@ -16248,7 +16563,7 @@
         <v>24</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="26" spans="2:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -16256,13 +16571,13 @@
         <v>18</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>1608</v>
+        <v>1622</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>1609</v>
+        <v>1623</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>1610</v>
+        <v>1624</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>98</v>
@@ -16284,7 +16599,7 @@
         <v>24</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="27" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -16292,13 +16607,13 @@
         <v>18</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>1611</v>
+        <v>1625</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>1612</v>
+        <v>1626</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>1629</v>
+        <v>1627</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>29</v>
@@ -16314,13 +16629,13 @@
         <v>-30</v>
       </c>
       <c r="J27" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K27" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K27" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L27" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="28" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -16328,13 +16643,13 @@
         <v>18</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>1620</v>
+        <v>1628</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>1613</v>
+        <v>1629</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>1621</v>
+        <v>1630</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>70</v>
@@ -16356,7 +16671,7 @@
         <v>24</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
       <c r="M28" s="3" t="s">
         <v>145</v>
@@ -16370,7 +16685,7 @@
         <v>1478</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>1614</v>
+        <v>1631</v>
       </c>
       <c r="E29" s="8" t="s">
         <v>1480</v>
@@ -16389,13 +16704,13 @@
         <v>660</v>
       </c>
       <c r="J29" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K29" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L29" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K29" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L29" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="30" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -16406,7 +16721,7 @@
         <v>1148</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>1615</v>
+        <v>1632</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>1150</v>
@@ -16431,7 +16746,7 @@
         <v>24</v>
       </c>
       <c r="L30" s="5" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="31" spans="2:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -16439,13 +16754,13 @@
         <v>18</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>1616</v>
+        <v>1633</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>1617</v>
+        <v>1634</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>1637</v>
+        <v>1635</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>131</v>
@@ -16461,13 +16776,13 @@
         <v>2675</v>
       </c>
       <c r="J31" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K31" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L31" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K31" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L31" s="8" t="s">
-        <v>1567</v>
       </c>
       <c r="M31" s="8" t="s">
         <v>145</v>
@@ -16478,13 +16793,13 @@
         <v>18</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>1618</v>
+        <v>1636</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>1619</v>
+        <v>1637</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>1635</v>
+        <v>1638</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>52</v>
@@ -16500,13 +16815,13 @@
         <v>1650</v>
       </c>
       <c r="J32" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K32" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L32" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K32" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L32" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="33" spans="2:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -16514,13 +16829,13 @@
         <v>18</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>1631</v>
+        <v>1639</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>1632</v>
+        <v>1640</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>1633</v>
+        <v>1641</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>85</v>
@@ -16536,13 +16851,13 @@
         <v>830</v>
       </c>
       <c r="J33" s="8" t="s">
+        <v>1569</v>
+      </c>
+      <c r="K33" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L33" s="8" t="s">
         <v>1566</v>
-      </c>
-      <c r="K33" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="L33" s="8" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="34" spans="2:17" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -16592,6 +16907,1579 @@
         <v>266</v>
       </c>
       <c r="Q34" s="11">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
+  <dimension ref="A1:Q43"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="49.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="76.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1642</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>1730</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>1731</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>1732</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="8">
+        <v>850</v>
+      </c>
+      <c r="H3" s="8">
+        <v>30</v>
+      </c>
+      <c r="I3" s="8">
+        <f t="shared" ref="I3:I42" si="0">G3-H3</f>
+        <v>820</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>1645</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>1646</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>1716</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G4" s="3">
+        <v>1500</v>
+      </c>
+      <c r="H4" s="3">
+        <v>30</v>
+      </c>
+      <c r="I4" s="3">
+        <f t="shared" si="0"/>
+        <v>1470</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>1727</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>1647</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>1728</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G5" s="6">
+        <v>4400</v>
+      </c>
+      <c r="H5" s="6">
+        <v>35</v>
+      </c>
+      <c r="I5" s="6">
+        <f t="shared" ref="I5" si="1">G5-H5</f>
+        <v>4365</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>1644</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>1648</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>1649</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>1714</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="3">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3">
+        <v>30</v>
+      </c>
+      <c r="I6" s="3">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>1650</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>1651</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>1742</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="8">
+        <v>470</v>
+      </c>
+      <c r="H7" s="8">
+        <v>30</v>
+      </c>
+      <c r="I7" s="8">
+        <f t="shared" si="0"/>
+        <v>440</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>1652</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>1653</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>1733</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="G8" s="8">
+        <v>0</v>
+      </c>
+      <c r="H8" s="8">
+        <v>25</v>
+      </c>
+      <c r="I8" s="8">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>1654</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>1655</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="8">
+        <v>850</v>
+      </c>
+      <c r="H9" s="8">
+        <v>30</v>
+      </c>
+      <c r="I9" s="8">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>966</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>1657</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>968</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="3">
+        <v>720</v>
+      </c>
+      <c r="H10" s="3">
+        <v>30</v>
+      </c>
+      <c r="I10" s="3">
+        <f t="shared" si="0"/>
+        <v>690</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>891</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>1658</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>1510</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="G11" s="8">
+        <v>915</v>
+      </c>
+      <c r="H11" s="8">
+        <v>25</v>
+      </c>
+      <c r="I11" s="8">
+        <f t="shared" si="0"/>
+        <v>890</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>1659</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>1660</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>1715</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="G12" s="3">
+        <v>510</v>
+      </c>
+      <c r="H12" s="3">
+        <v>20</v>
+      </c>
+      <c r="I12" s="3">
+        <f t="shared" si="0"/>
+        <v>490</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>1661</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>1662</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>1663</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="3">
+        <v>0</v>
+      </c>
+      <c r="H13" s="3">
+        <v>25</v>
+      </c>
+      <c r="I13" s="3">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>1664</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>1665</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>1723</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="G14" s="6">
+        <v>515</v>
+      </c>
+      <c r="H14" s="6">
+        <v>25</v>
+      </c>
+      <c r="I14" s="6">
+        <f t="shared" si="0"/>
+        <v>490</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>1666</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>1667</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>1668</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G15" s="6">
+        <v>895</v>
+      </c>
+      <c r="H15" s="6">
+        <v>25</v>
+      </c>
+      <c r="I15" s="6">
+        <f t="shared" si="0"/>
+        <v>870</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>1225</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>1722</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>1227</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="G16" s="6">
+        <v>710</v>
+      </c>
+      <c r="H16" s="6">
+        <v>20</v>
+      </c>
+      <c r="I16" s="6">
+        <f t="shared" si="0"/>
+        <v>690</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>1725</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>1669</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>1670</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="G17" s="6">
+        <v>515</v>
+      </c>
+      <c r="H17" s="6">
+        <v>25</v>
+      </c>
+      <c r="I17" s="6">
+        <f t="shared" si="0"/>
+        <v>490</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>1671</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>1672</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>1734</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="G18" s="8">
+        <v>1855</v>
+      </c>
+      <c r="H18" s="8">
+        <v>25</v>
+      </c>
+      <c r="I18" s="8">
+        <f t="shared" si="0"/>
+        <v>1830</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K18" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>1673</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>1674</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>1675</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="G19" s="8">
+        <v>795</v>
+      </c>
+      <c r="H19" s="8">
+        <v>25</v>
+      </c>
+      <c r="I19" s="8">
+        <f t="shared" si="0"/>
+        <v>770</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>1676</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>1677</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>1678</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G20" s="6">
+        <v>0</v>
+      </c>
+      <c r="H20" s="6">
+        <v>25</v>
+      </c>
+      <c r="I20" s="6">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>1680</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>1717</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G21" s="3">
+        <v>850</v>
+      </c>
+      <c r="H21" s="3">
+        <v>30</v>
+      </c>
+      <c r="I21" s="3">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>1737</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>1681</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>1682</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G22" s="8">
+        <v>1120</v>
+      </c>
+      <c r="H22" s="8">
+        <v>30</v>
+      </c>
+      <c r="I22" s="8">
+        <f t="shared" si="0"/>
+        <v>1090</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>1683</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>1684</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>1743</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="G23" s="8">
+        <v>0</v>
+      </c>
+      <c r="H23" s="8">
+        <v>25</v>
+      </c>
+      <c r="I23" s="8">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>1332</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>1685</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>1334</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>1335</v>
+      </c>
+      <c r="G24" s="8">
+        <v>775</v>
+      </c>
+      <c r="H24" s="8">
+        <v>35</v>
+      </c>
+      <c r="I24" s="8">
+        <f t="shared" si="0"/>
+        <v>740</v>
+      </c>
+      <c r="J24" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K24" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>1686</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>1687</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>1724</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G25" s="6">
+        <v>915</v>
+      </c>
+      <c r="H25" s="6">
+        <v>25</v>
+      </c>
+      <c r="I25" s="6">
+        <f t="shared" si="0"/>
+        <v>890</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>1688</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>1713</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G26" s="3">
+        <v>520</v>
+      </c>
+      <c r="H26" s="3">
+        <v>30</v>
+      </c>
+      <c r="I26" s="3">
+        <f t="shared" si="0"/>
+        <v>490</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>1267</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>1689</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>1269</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G27" s="8">
+        <v>710</v>
+      </c>
+      <c r="H27" s="8">
+        <v>30</v>
+      </c>
+      <c r="I27" s="8">
+        <f t="shared" si="0"/>
+        <v>680</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K27" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>1690</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>1691</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>1735</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="G28" s="8">
+        <v>520</v>
+      </c>
+      <c r="H28" s="8">
+        <v>30</v>
+      </c>
+      <c r="I28" s="8">
+        <f t="shared" si="0"/>
+        <v>490</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K28" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L28" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>1739</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>1741</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>1740</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G29" s="8">
+        <v>0</v>
+      </c>
+      <c r="H29" s="8">
+        <v>30</v>
+      </c>
+      <c r="I29" s="8">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J29" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K29" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L29" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>1692</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>1693</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>1694</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="G30" s="3">
+        <v>800</v>
+      </c>
+      <c r="H30" s="3">
+        <v>20</v>
+      </c>
+      <c r="I30" s="3">
+        <f t="shared" si="0"/>
+        <v>780</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L30" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>1695</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>1696</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>1736</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="G31" s="8">
+        <v>0</v>
+      </c>
+      <c r="H31" s="8">
+        <v>25</v>
+      </c>
+      <c r="I31" s="8">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K31" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L31" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>1697</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>1698</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>1738</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="G32" s="8">
+        <v>520</v>
+      </c>
+      <c r="H32" s="8">
+        <v>30</v>
+      </c>
+      <c r="I32" s="8">
+        <f t="shared" si="0"/>
+        <v>490</v>
+      </c>
+      <c r="J32" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K32" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L32" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>1700</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G33" s="3">
+        <v>0</v>
+      </c>
+      <c r="H33" s="3">
+        <v>25</v>
+      </c>
+      <c r="I33" s="3">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J33" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L33" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>1720</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>1701</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>1721</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="G34" s="3">
+        <v>850</v>
+      </c>
+      <c r="H34" s="3">
+        <v>20</v>
+      </c>
+      <c r="I34" s="3">
+        <f t="shared" si="0"/>
+        <v>830</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L34" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>1267</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>1702</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>1729</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="G35" s="8">
+        <v>990</v>
+      </c>
+      <c r="H35" s="8">
+        <v>30</v>
+      </c>
+      <c r="I35" s="8">
+        <f t="shared" si="0"/>
+        <v>960</v>
+      </c>
+      <c r="J35" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K35" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L35" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>1703</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>1704</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>1705</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G36" s="3">
+        <v>0</v>
+      </c>
+      <c r="H36" s="3">
+        <v>25</v>
+      </c>
+      <c r="I36" s="3">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>1706</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>1707</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>1708</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G37" s="8">
+        <v>1020</v>
+      </c>
+      <c r="H37" s="8">
+        <v>30</v>
+      </c>
+      <c r="I37" s="8">
+        <f t="shared" si="0"/>
+        <v>990</v>
+      </c>
+      <c r="J37" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K37" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L37" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>1709</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>1710</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>1711</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G38" s="8">
+        <v>860</v>
+      </c>
+      <c r="H38" s="8">
+        <v>30</v>
+      </c>
+      <c r="I38" s="8">
+        <f t="shared" si="0"/>
+        <v>830</v>
+      </c>
+      <c r="J38" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K38" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L38" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>1712</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>1726</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G39" s="6">
+        <v>30</v>
+      </c>
+      <c r="H39" s="6">
+        <v>30</v>
+      </c>
+      <c r="I39" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L39" s="6" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>953</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="G40" s="8">
+        <v>30</v>
+      </c>
+      <c r="H40" s="8">
+        <v>30</v>
+      </c>
+      <c r="I40" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J40" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="K40" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L40" s="8" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G41" s="3">
+        <v>0</v>
+      </c>
+      <c r="H41" s="3">
+        <v>40</v>
+      </c>
+      <c r="I41" s="3">
+        <f t="shared" si="0"/>
+        <v>-40</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K41" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L41" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>1718</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>1719</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G42" s="3">
+        <v>0</v>
+      </c>
+      <c r="H42" s="3">
+        <v>30</v>
+      </c>
+      <c r="I42" s="3">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K42" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L42" s="3" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>1136</v>
+      </c>
+      <c r="D43" s="15" t="s">
+        <v>1744</v>
+      </c>
+      <c r="E43" s="15" t="s">
+        <v>1138</v>
+      </c>
+      <c r="F43" s="16">
+        <v>7</v>
+      </c>
+      <c r="G43" s="16">
+        <v>810</v>
+      </c>
+      <c r="H43" s="16">
+        <v>30</v>
+      </c>
+      <c r="I43" s="16">
+        <f>G43-H43</f>
+        <v>780</v>
+      </c>
+      <c r="J43" s="15" t="s">
+        <v>1131</v>
+      </c>
+      <c r="K43" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="L43" s="15" t="s">
+        <v>1124</v>
+      </c>
+      <c r="M43" s="17" t="s">
+        <v>264</v>
+      </c>
+      <c r="N43" s="17" t="s">
+        <v>265</v>
+      </c>
+      <c r="O43" s="17" t="s">
+        <v>265</v>
+      </c>
+      <c r="P43" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="Q43" s="15">
         <v>1</v>
       </c>
     </row>
@@ -18892,7 +20780,7 @@
         <v>30</v>
       </c>
       <c r="I35" s="6">
-        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I55" si="1">G35-H35</f>
         <v>2090</v>
       </c>
       <c r="J35" s="6" t="s">
@@ -26075,7 +27963,7 @@
         <v>30</v>
       </c>
       <c r="I35" s="8">
-        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I58" si="1">G35-H35</f>
         <v>-30</v>
       </c>
       <c r="J35" s="8" t="s">

</xml_diff>

<commit_message>
Update don tra logic function
</commit_message>
<xml_diff>
--- a/data/May/Data_May.xlsx
+++ b/data/May/Data_May.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\May\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5DF3EDC-0EFD-4B8D-B6CA-60663BD1634D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1EFE784-8CA9-4FA5-BC8A-D6340B12189F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01-05" sheetId="4" r:id="rId1"/>
@@ -35,6 +35,7 @@
     <sheet name="25-05" sheetId="24" r:id="rId20"/>
     <sheet name="26-05" sheetId="25" r:id="rId21"/>
     <sheet name="27-05" sheetId="26" r:id="rId22"/>
+    <sheet name="28-05" sheetId="27" r:id="rId23"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -57,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6814" uniqueCount="2113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7053" uniqueCount="2183">
   <si>
     <t>THU 6</t>
   </si>
@@ -6227,60 +6228,72 @@
     <t>Nhận hộ fb Nguyễn Hà</t>
   </si>
   <si>
+    <t>HD023711</t>
+  </si>
+  <si>
+    <t>27-05-2026</t>
+  </si>
+  <si>
+    <t>Thúy Nguyễn</t>
+  </si>
+  <si>
+    <t>HD023794</t>
+  </si>
+  <si>
+    <t>598/10 điện biên phủ, p.22</t>
+  </si>
+  <si>
+    <t>ng nhận QP</t>
+  </si>
+  <si>
+    <t>HD023827</t>
+  </si>
+  <si>
+    <t>số 28 khu kdc nam long thạnh lộc</t>
+  </si>
+  <si>
+    <t>HUYỀN NGUYỄN</t>
+  </si>
+  <si>
+    <t>HD023936</t>
+  </si>
+  <si>
+    <t>Số 8 Ba Vì, P4</t>
+  </si>
+  <si>
+    <t>Giang Phạm</t>
+  </si>
+  <si>
+    <t>HD023787</t>
+  </si>
+  <si>
+    <t>136 hoàng hoa thám, p7</t>
+  </si>
+  <si>
+    <t>HD023906</t>
+  </si>
+  <si>
+    <t>77-89 nam kỳ khởi nghĩa bến thành</t>
+  </si>
+  <si>
+    <t>KimVy Phương Anh</t>
+  </si>
+  <si>
+    <t>HD023841</t>
+  </si>
+  <si>
+    <t>214/B14A nguyễn trãi, cầu ông lãnh</t>
+  </si>
+  <si>
+    <t>HD023837</t>
+  </si>
+  <si>
+    <t>Can 32.07 - the Pegasuite 1- số 1002 tạ quang bửu, phường 5</t>
+  </si>
+  <si>
     <t>AT 27-05</t>
   </si>
   <si>
-    <t>27-05-2026</t>
-  </si>
-  <si>
-    <t>HD023794</t>
-  </si>
-  <si>
-    <t>ng nhận QP</t>
-  </si>
-  <si>
-    <t>HD023827</t>
-  </si>
-  <si>
-    <t>số 28 khu kdc nam long thạnh lộc</t>
-  </si>
-  <si>
-    <t>HUYỀN NGUYỄN</t>
-  </si>
-  <si>
-    <t>HD023936</t>
-  </si>
-  <si>
-    <t>Giang Phạm</t>
-  </si>
-  <si>
-    <t>HD023787</t>
-  </si>
-  <si>
-    <t>136 hoàng hoa thám, p7</t>
-  </si>
-  <si>
-    <t>HD023906</t>
-  </si>
-  <si>
-    <t>77-89 nam kỳ khởi nghĩa bến thành</t>
-  </si>
-  <si>
-    <t>KimVy Phương Anh</t>
-  </si>
-  <si>
-    <t>HD023841</t>
-  </si>
-  <si>
-    <t>214/B14A nguyễn trãi, cầu ông lãnh</t>
-  </si>
-  <si>
-    <t>HD023837</t>
-  </si>
-  <si>
-    <t>Can 32.07 - the Pegasuite 1- số 1002 tạ quang bửu, phường 5</t>
-  </si>
-  <si>
     <t>HD023572</t>
   </si>
   <si>
@@ -6314,6 +6327,12 @@
     <t>Thiên An</t>
   </si>
   <si>
+    <t>HD023884</t>
+  </si>
+  <si>
+    <t>D aqua 301 bình động, phú định</t>
+  </si>
+  <si>
     <t>Thao Thanh Nguyen</t>
   </si>
   <si>
@@ -6326,6 +6345,12 @@
     <t>S$3164-Mrskill)</t>
   </si>
   <si>
+    <t>HD022602</t>
+  </si>
+  <si>
+    <t>674 đường số 2, Phường 13</t>
+  </si>
+  <si>
     <t>Khánh Như</t>
   </si>
   <si>
@@ -6335,6 +6360,9 @@
     <t>688/23/1c Hương Lộ 2, phường Bình Trị Đông A</t>
   </si>
   <si>
+    <t>GIA HUY nhận hộ ELIS NGUYỄN (singapore)</t>
+  </si>
+  <si>
     <t>HD023838</t>
   </si>
   <si>
@@ -6344,58 +6372,241 @@
     <t>HD023850</t>
   </si>
   <si>
+    <t>1041/80/3/5 trần xuân soạn phường tân hưng</t>
+  </si>
+  <si>
     <t>cô Loan fb Trịnh Trâm</t>
   </si>
   <si>
     <t>HD023930</t>
   </si>
   <si>
+    <t>124/18/12 võ văn hát p long trường</t>
+  </si>
+  <si>
     <t>NHƯ THẢO</t>
   </si>
   <si>
+    <t>259 đường 9a kdc Trung Sơn, Bình Hưng</t>
+  </si>
+  <si>
     <t>Ellie Quach</t>
   </si>
   <si>
+    <t>8A Sông thương, Phường 2</t>
+  </si>
+  <si>
     <t>SỈ HƯƠNG TRẦN</t>
   </si>
   <si>
-    <t>HD023711</t>
-  </si>
-  <si>
-    <t>Thúy Nguyễn</t>
-  </si>
-  <si>
-    <t>598/10 điện biên phủ, p.22</t>
-  </si>
-  <si>
-    <t>8A Sông thương, Phường 2</t>
-  </si>
-  <si>
-    <t>GIA HUY nhận hộ ELIS NGUYỄN (singapore)</t>
-  </si>
-  <si>
-    <t>Số 8 Ba Vì, P4</t>
-  </si>
-  <si>
-    <t>259 đường 9a kdc Trung Sơn, Bình Hưng</t>
-  </si>
-  <si>
-    <t>HD022602</t>
-  </si>
-  <si>
-    <t>674 đường số 2, Phường 13</t>
-  </si>
-  <si>
-    <t>124/18/12 võ văn hát p long trường</t>
-  </si>
-  <si>
-    <t>1041/80/3/5 trần xuân soạn phường tân hưng</t>
-  </si>
-  <si>
-    <t>HD023884</t>
-  </si>
-  <si>
-    <t>D aqua 301 bình động, phú định</t>
+    <t>NGAY 28-5</t>
+  </si>
+  <si>
+    <t>Uyên Trần</t>
+  </si>
+  <si>
+    <t>HD024168</t>
+  </si>
+  <si>
+    <t>AT 28-05</t>
+  </si>
+  <si>
+    <t>28-05-2026</t>
+  </si>
+  <si>
+    <t>Thanh Vy</t>
+  </si>
+  <si>
+    <t>HD024163</t>
+  </si>
+  <si>
+    <t>Thảo My</t>
+  </si>
+  <si>
+    <t>HD024170</t>
+  </si>
+  <si>
+    <t>HD024033</t>
+  </si>
+  <si>
+    <t>Kelly Phan</t>
+  </si>
+  <si>
+    <t>HD024129</t>
+  </si>
+  <si>
+    <t>Tuệ Nhi</t>
+  </si>
+  <si>
+    <t>HD024045</t>
+  </si>
+  <si>
+    <t>92-94 nam kỳ khởi nghĩa- bến nghé</t>
+  </si>
+  <si>
+    <t>HD024006</t>
+  </si>
+  <si>
+    <t>24 Lê Thánh Tôn (BIDV), P.Bến Nghé</t>
+  </si>
+  <si>
+    <t>Linh fb Phan Thị Tuyết Nhung</t>
+  </si>
+  <si>
+    <t>HD023982</t>
+  </si>
+  <si>
+    <t>Nguyễn Châu Tuệ Lâm</t>
+  </si>
+  <si>
+    <t>HD024027</t>
+  </si>
+  <si>
+    <t>74/1h ds9 linh trung</t>
+  </si>
+  <si>
+    <t>Ngân</t>
+  </si>
+  <si>
+    <t>HD023968</t>
+  </si>
+  <si>
+    <t>Toà A2 Alnata diamond đường N1 Tân Sơn Nhì</t>
+  </si>
+  <si>
+    <t>HD024142</t>
+  </si>
+  <si>
+    <t>HD024157</t>
+  </si>
+  <si>
+    <t>HD023918</t>
+  </si>
+  <si>
+    <t>Minh Thư nhận hộ ( water) fb Thuỷ Vũ</t>
+  </si>
+  <si>
+    <t>HD024179</t>
+  </si>
+  <si>
+    <t>22, TÂN THỚI NHẤT 1B, Phường Tân Thới Nhất</t>
+  </si>
+  <si>
+    <t>Tất Phú</t>
+  </si>
+  <si>
+    <t>HD023941</t>
+  </si>
+  <si>
+    <t>Bệnh viện Nhi đồng 1: 532 Lý Thái Tổ, P10</t>
+  </si>
+  <si>
+    <t>HD24001</t>
+  </si>
+  <si>
+    <t>Trần Lan</t>
+  </si>
+  <si>
+    <t>HD024017</t>
+  </si>
+  <si>
+    <t>Cô Kiều Hương fb Vân Trần</t>
+  </si>
+  <si>
+    <t>HD023954</t>
+  </si>
+  <si>
+    <t>168A Trần Huy Liệu Phường 15</t>
+  </si>
+  <si>
+    <t>HD023966</t>
+  </si>
+  <si>
+    <t>12 nguyễn công trứ, thái bình</t>
+  </si>
+  <si>
+    <t>phạm minh phi_F3: Theer To Lao</t>
+  </si>
+  <si>
+    <t>Diễm Phúc</t>
+  </si>
+  <si>
+    <t>HD024175</t>
+  </si>
+  <si>
+    <t>314/138 đường âu dương lân, p3</t>
+  </si>
+  <si>
+    <t>Đậu Đậu</t>
+  </si>
+  <si>
+    <t>HD024181</t>
+  </si>
+  <si>
+    <t>106/4 phan van tri phường 12</t>
+  </si>
+  <si>
+    <t>HD024164</t>
+  </si>
+  <si>
+    <t>Linh Nga Anna</t>
+  </si>
+  <si>
+    <t>khả trinh</t>
+  </si>
+  <si>
+    <t>82/17/20đinh tiên hoàng p1</t>
+  </si>
+  <si>
+    <t>chị hương fb Kim Tien Pham</t>
+  </si>
+  <si>
+    <t>HD024093</t>
+  </si>
+  <si>
+    <t>33 đường số 6 p26</t>
+  </si>
+  <si>
+    <t>190 võ văn ngân</t>
+  </si>
+  <si>
+    <t>HD023972</t>
+  </si>
+  <si>
+    <t>433/11, Lê Đức Thọ, Phường 17</t>
+  </si>
+  <si>
+    <t>201 Đường Hoàng Hoa Thám, Phường 13</t>
+  </si>
+  <si>
+    <t>Nguyễn Trinh</t>
+  </si>
+  <si>
+    <t>29/10c trần thái tông</t>
+  </si>
+  <si>
+    <t>Toà Aster - Urbun Green (đối diện Vạn Phúc)</t>
+  </si>
+  <si>
+    <t>91/12 nguyễn thanh tuyền p1</t>
+  </si>
+  <si>
+    <t>240/6A lê thánh tôn phường bến thành</t>
+  </si>
+  <si>
+    <t>Thủy Heri</t>
+  </si>
+  <si>
+    <t>HD024145</t>
+  </si>
+  <si>
+    <t>184/17/35 bãi sậy phường bình tiên</t>
+  </si>
+  <si>
+    <t>137/84D âu dương lân - p2</t>
+  </si>
+  <si>
+    <t>20B Trần Văn Quang, Phường Bảy Hiền</t>
   </si>
 </sst>
 </file>
@@ -8040,7 +8251,7 @@
         <v>30</v>
       </c>
       <c r="I35" s="6">
-        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I56" si="1">G35-H35</f>
         <v>30</v>
       </c>
       <c r="J35" s="6" t="s">
@@ -23996,7 +24207,7 @@
         <v>25</v>
       </c>
       <c r="I35" s="3">
-        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I55" si="1">G35-H35</f>
         <v>700</v>
       </c>
       <c r="J35" s="3" t="s">
@@ -25914,10 +26125,12 @@
   <dimension ref="A1:P26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
     <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="55" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
     <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -25991,7 +26204,7 @@
         <v>2055</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>2100</v>
+        <v>2056</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>1313</v>
@@ -26024,13 +26237,13 @@
         <v>18</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>2101</v>
+        <v>2058</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>2058</v>
+        <v>2059</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>2102</v>
+        <v>2060</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>81</v>
@@ -26060,13 +26273,13 @@
         <v>18</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>2059</v>
+        <v>2061</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>2060</v>
+        <v>2062</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>2061</v>
+        <v>2063</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>29</v>
@@ -26096,13 +26309,13 @@
         <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>2062</v>
+        <v>2064</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>2063</v>
+        <v>2065</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>2105</v>
+        <v>2066</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>102</v>
@@ -26132,13 +26345,13 @@
         <v>18</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>2064</v>
+        <v>2067</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>2065</v>
+        <v>2068</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>2066</v>
+        <v>2069</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>81</v>
@@ -26171,10 +26384,10 @@
         <v>593</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>2067</v>
+        <v>2070</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>2068</v>
+        <v>2071</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>63</v>
@@ -26204,13 +26417,13 @@
         <v>18</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>2069</v>
+        <v>2072</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>2070</v>
+        <v>2073</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>2071</v>
+        <v>2074</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>63</v>
@@ -26243,10 +26456,10 @@
         <v>1754</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>2072</v>
+        <v>2075</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>2073</v>
+        <v>2076</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>41</v>
@@ -26262,7 +26475,7 @@
         <v>780</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>2056</v>
+        <v>2077</v>
       </c>
       <c r="K10" s="8" t="s">
         <v>24</v>
@@ -26279,7 +26492,7 @@
         <v>1411</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>2074</v>
+        <v>2078</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>763</v>
@@ -26298,7 +26511,7 @@
         <v>-30</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>2056</v>
+        <v>2077</v>
       </c>
       <c r="K11" s="8" t="s">
         <v>24</v>
@@ -26315,7 +26528,7 @@
         <v>1442</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>2075</v>
+        <v>2079</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>1444</v>
@@ -26334,7 +26547,7 @@
         <v>-30</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>2056</v>
+        <v>2077</v>
       </c>
       <c r="K12" s="8" t="s">
         <v>24</v>
@@ -26351,10 +26564,10 @@
         <v>1917</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>2076</v>
+        <v>2080</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>2077</v>
+        <v>2081</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>85</v>
@@ -26370,7 +26583,7 @@
         <v>-25</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>2056</v>
+        <v>2077</v>
       </c>
       <c r="K13" s="8" t="s">
         <v>24</v>
@@ -26384,13 +26597,13 @@
         <v>18</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>2078</v>
+        <v>2082</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>2079</v>
+        <v>2083</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>2080</v>
+        <v>2084</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>41</v>
@@ -26406,7 +26619,7 @@
         <v>440</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>2056</v>
+        <v>2077</v>
       </c>
       <c r="K14" s="8" t="s">
         <v>24</v>
@@ -26420,13 +26633,13 @@
         <v>18</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>2081</v>
+        <v>2085</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>2082</v>
+        <v>2086</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>2083</v>
+        <v>2087</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>29</v>
@@ -26456,13 +26669,13 @@
         <v>18</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>2084</v>
+        <v>2088</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>2111</v>
+        <v>2089</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>2112</v>
+        <v>2090</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>41</v>
@@ -26478,7 +26691,7 @@
         <v>710</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>2056</v>
+        <v>2077</v>
       </c>
       <c r="K16" s="8" t="s">
         <v>24</v>
@@ -26495,13 +26708,13 @@
         <v>18</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>2085</v>
+        <v>2091</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>2086</v>
+        <v>2092</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>2087</v>
+        <v>2093</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>63</v>
@@ -26531,13 +26744,13 @@
         <v>18</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>2088</v>
+        <v>2094</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>2107</v>
+        <v>2095</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>2108</v>
+        <v>2096</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>127</v>
@@ -26553,7 +26766,7 @@
         <v>-25</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>2056</v>
+        <v>2077</v>
       </c>
       <c r="K18" s="8" t="s">
         <v>24</v>
@@ -26567,13 +26780,13 @@
         <v>18</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>2089</v>
+        <v>2097</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>2090</v>
+        <v>2098</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>2091</v>
+        <v>2099</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>22</v>
@@ -26589,7 +26802,7 @@
         <v>820</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>2056</v>
+        <v>2077</v>
       </c>
       <c r="K19" s="8" t="s">
         <v>24</v>
@@ -26603,10 +26816,10 @@
         <v>18</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>2104</v>
+        <v>2100</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>2092</v>
+        <v>2101</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>1415</v>
@@ -26639,13 +26852,13 @@
         <v>18</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>2093</v>
+        <v>2102</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>2094</v>
+        <v>2103</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>2110</v>
+        <v>2104</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>131</v>
@@ -26661,7 +26874,7 @@
         <v>790</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>2056</v>
+        <v>2077</v>
       </c>
       <c r="K21" s="8" t="s">
         <v>24</v>
@@ -26675,13 +26888,13 @@
         <v>18</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>2095</v>
+        <v>2105</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>2096</v>
+        <v>2106</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>2109</v>
+        <v>2107</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>149</v>
@@ -26697,7 +26910,7 @@
         <v>890</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>2056</v>
+        <v>2077</v>
       </c>
       <c r="K22" s="8" t="s">
         <v>24</v>
@@ -26714,10 +26927,10 @@
         <v>18</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>2097</v>
+        <v>2108</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>2106</v>
+        <v>2109</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>52</v>
@@ -26733,7 +26946,7 @@
         <v>660</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>2056</v>
+        <v>2077</v>
       </c>
       <c r="K23" s="8" t="s">
         <v>24</v>
@@ -26786,10 +26999,10 @@
         <v>18</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>2098</v>
+        <v>2110</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>2103</v>
+        <v>2111</v>
       </c>
       <c r="F25" s="6" t="s">
         <v>102</v>
@@ -26822,7 +27035,7 @@
         <v>18</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>2099</v>
+        <v>2112</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>952</v>
@@ -26852,6 +27065,1078 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
+  <dimension ref="A1:Q29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="42.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>2114</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>2115</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>2181</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="8">
+        <v>720</v>
+      </c>
+      <c r="H3" s="8">
+        <v>30</v>
+      </c>
+      <c r="I3" s="8">
+        <f t="shared" ref="I3:I28" si="0">G3-H3</f>
+        <v>690</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>2116</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>2118</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>2119</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>2182</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="G4" s="8">
+        <v>1165</v>
+      </c>
+      <c r="H4" s="8">
+        <v>25</v>
+      </c>
+      <c r="I4" s="8">
+        <f t="shared" si="0"/>
+        <v>1140</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>2116</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>2120</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>2121</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>2176</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G5" s="6">
+        <v>915</v>
+      </c>
+      <c r="H5" s="6">
+        <v>25</v>
+      </c>
+      <c r="I5" s="6">
+        <f t="shared" si="0"/>
+        <v>890</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>2164</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>2122</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>2165</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G6" s="3">
+        <v>900</v>
+      </c>
+      <c r="H6" s="3">
+        <v>20</v>
+      </c>
+      <c r="I6" s="3">
+        <f t="shared" si="0"/>
+        <v>880</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>2123</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>2124</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>2177</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G7" s="6">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6">
+        <v>25</v>
+      </c>
+      <c r="I7" s="6">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>2125</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>2126</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>2127</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" s="6">
+        <v>0</v>
+      </c>
+      <c r="H8" s="6">
+        <v>25</v>
+      </c>
+      <c r="I8" s="6">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>1633</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>2128</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>2129</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6">
+        <v>25</v>
+      </c>
+      <c r="I9" s="6">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>2178</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>2179</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>2180</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="G10" s="8">
+        <v>0</v>
+      </c>
+      <c r="H10" s="8">
+        <v>25</v>
+      </c>
+      <c r="I10" s="8">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>2116</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="8" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>2130</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>2131</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>2172</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G11" s="3">
+        <v>0</v>
+      </c>
+      <c r="H11" s="3">
+        <v>25</v>
+      </c>
+      <c r="I11" s="3">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>2132</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>2133</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>2134</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" s="3">
+        <v>3650</v>
+      </c>
+      <c r="H12" s="3">
+        <v>40</v>
+      </c>
+      <c r="I12" s="3">
+        <f t="shared" si="0"/>
+        <v>3610</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>2117</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>2135</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>2136</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>2137</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13" s="8">
+        <v>845</v>
+      </c>
+      <c r="H13" s="8">
+        <v>25</v>
+      </c>
+      <c r="I13" s="8">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>2116</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="8" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>2085</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>2138</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>2087</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" s="3">
+        <v>0</v>
+      </c>
+      <c r="H14" s="3">
+        <v>30</v>
+      </c>
+      <c r="I14" s="3">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>2173</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>2139</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>2174</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G15" s="3">
+        <v>775</v>
+      </c>
+      <c r="H15" s="3">
+        <v>25</v>
+      </c>
+      <c r="I15" s="3">
+        <f t="shared" si="0"/>
+        <v>750</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>1930</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>2140</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>1932</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16" s="8">
+        <v>850</v>
+      </c>
+      <c r="H16" s="8">
+        <v>30</v>
+      </c>
+      <c r="I16" s="8">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>2116</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="8" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>2141</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>2142</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>2143</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G17" s="3">
+        <v>0</v>
+      </c>
+      <c r="H17" s="3">
+        <v>30</v>
+      </c>
+      <c r="I17" s="3">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>2144</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>2145</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>2146</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="G18" s="6">
+        <v>595</v>
+      </c>
+      <c r="H18" s="6">
+        <v>25</v>
+      </c>
+      <c r="I18" s="6">
+        <f t="shared" si="0"/>
+        <v>570</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>2170</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>2171</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G19" s="3">
+        <v>1775</v>
+      </c>
+      <c r="H19" s="3">
+        <v>25</v>
+      </c>
+      <c r="I19" s="3">
+        <f t="shared" si="0"/>
+        <v>1750</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>2166</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>2147</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G20" s="3">
+        <v>0</v>
+      </c>
+      <c r="H20" s="3">
+        <v>25</v>
+      </c>
+      <c r="I20" s="3">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>2148</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>2149</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>2169</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G21" s="3">
+        <v>1120</v>
+      </c>
+      <c r="H21" s="3">
+        <v>30</v>
+      </c>
+      <c r="I21" s="3">
+        <f t="shared" si="0"/>
+        <v>1090</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>2150</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>2151</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>2152</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="G22" s="6">
+        <v>970</v>
+      </c>
+      <c r="H22" s="6">
+        <v>20</v>
+      </c>
+      <c r="I22" s="6">
+        <f t="shared" si="0"/>
+        <v>950</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>2153</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>2154</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G23" s="6">
+        <v>845</v>
+      </c>
+      <c r="H23" s="6">
+        <v>25</v>
+      </c>
+      <c r="I23" s="6">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>2155</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>2167</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>2168</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G24" s="3">
+        <v>1720</v>
+      </c>
+      <c r="H24" s="3">
+        <v>20</v>
+      </c>
+      <c r="I24" s="3">
+        <f t="shared" si="0"/>
+        <v>1700</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>2156</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>2157</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>2158</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G25" s="8">
+        <v>850</v>
+      </c>
+      <c r="H25" s="8">
+        <v>30</v>
+      </c>
+      <c r="I25" s="8">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>2116</v>
+      </c>
+      <c r="K25" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="8" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>2159</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>2160</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>2161</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G26" s="3">
+        <v>0</v>
+      </c>
+      <c r="H26" s="3">
+        <v>20</v>
+      </c>
+      <c r="I26" s="3">
+        <f t="shared" si="0"/>
+        <v>-20</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>2117</v>
+      </c>
+      <c r="M26" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>2162</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>2175</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G27" s="3">
+        <v>860</v>
+      </c>
+      <c r="H27" s="3">
+        <v>30</v>
+      </c>
+      <c r="I27" s="3">
+        <f t="shared" si="0"/>
+        <v>830</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>2163</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>2087</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0</v>
+      </c>
+      <c r="H28" s="3">
+        <v>60</v>
+      </c>
+      <c r="I28" s="3">
+        <f t="shared" si="0"/>
+        <v>-60</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>1887</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>1888</v>
+      </c>
+      <c r="E29" s="11" t="s">
+        <v>1889</v>
+      </c>
+      <c r="F29" s="12">
+        <v>4</v>
+      </c>
+      <c r="G29" s="11">
+        <v>845</v>
+      </c>
+      <c r="H29" s="11">
+        <v>25</v>
+      </c>
+      <c r="I29" s="11">
+        <v>820</v>
+      </c>
+      <c r="J29" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="K29" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="L29" s="11" t="s">
+        <v>1873</v>
+      </c>
+      <c r="M29" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="N29" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="O29" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="P29" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="Q29" s="11">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -28132,7 +29417,7 @@
         <v>30</v>
       </c>
       <c r="I35" s="6">
-        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I55" si="1">G35-H35</f>
         <v>2090</v>
       </c>
       <c r="J35" s="6" t="s">
@@ -35315,7 +36600,7 @@
         <v>30</v>
       </c>
       <c r="I35" s="8">
-        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I58" si="1">G35-H35</f>
         <v>-30</v>
       </c>
       <c r="J35" s="8" t="s">

</xml_diff>

<commit_message>
Update Jun excel template
</commit_message>
<xml_diff>
--- a/data/May/Data_May.xlsx
+++ b/data/May/Data_May.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\May\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1EFE784-8CA9-4FA5-BC8A-D6340B12189F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1466695-D300-4D95-8388-7E8787C37A8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="24" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01-05" sheetId="4" r:id="rId1"/>
@@ -36,6 +36,8 @@
     <sheet name="26-05" sheetId="25" r:id="rId21"/>
     <sheet name="27-05" sheetId="26" r:id="rId22"/>
     <sheet name="28-05" sheetId="27" r:id="rId23"/>
+    <sheet name="29-05" sheetId="28" r:id="rId24"/>
+    <sheet name="30-05" sheetId="29" r:id="rId25"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -58,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7053" uniqueCount="2183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7503" uniqueCount="2320">
   <si>
     <t>THU 6</t>
   </si>
@@ -6408,6 +6410,9 @@
     <t>HD024168</t>
   </si>
   <si>
+    <t>137/84D âu dương lân - p2</t>
+  </si>
+  <si>
     <t>AT 28-05</t>
   </si>
   <si>
@@ -6420,21 +6425,36 @@
     <t>HD024163</t>
   </si>
   <si>
+    <t>20B Trần Văn Quang, Phường Bảy Hiền</t>
+  </si>
+  <si>
     <t>Thảo My</t>
   </si>
   <si>
     <t>HD024170</t>
   </si>
   <si>
+    <t>91/12 nguyễn thanh tuyền p1</t>
+  </si>
+  <si>
+    <t>khả trinh</t>
+  </si>
+  <si>
     <t>HD024033</t>
   </si>
   <si>
+    <t>82/17/20đinh tiên hoàng p1</t>
+  </si>
+  <si>
     <t>Kelly Phan</t>
   </si>
   <si>
     <t>HD024129</t>
   </si>
   <si>
+    <t>240/6A lê thánh tôn phường bến thành</t>
+  </si>
+  <si>
     <t>Tuệ Nhi</t>
   </si>
   <si>
@@ -6450,12 +6470,24 @@
     <t>24 Lê Thánh Tôn (BIDV), P.Bến Nghé</t>
   </si>
   <si>
+    <t>Thủy Heri</t>
+  </si>
+  <si>
+    <t>HD024145</t>
+  </si>
+  <si>
+    <t>184/17/35 bãi sậy phường bình tiên</t>
+  </si>
+  <si>
     <t>Linh fb Phan Thị Tuyết Nhung</t>
   </si>
   <si>
     <t>HD023982</t>
   </si>
   <si>
+    <t>201 Đường Hoàng Hoa Thám, Phường 13</t>
+  </si>
+  <si>
     <t>Nguyễn Châu Tuệ Lâm</t>
   </si>
   <si>
@@ -6477,9 +6509,15 @@
     <t>HD024142</t>
   </si>
   <si>
+    <t>Nguyễn Trinh</t>
+  </si>
+  <si>
     <t>HD024157</t>
   </si>
   <si>
+    <t>29/10c trần thái tông</t>
+  </si>
+  <si>
     <t>HD023918</t>
   </si>
   <si>
@@ -6501,6 +6539,15 @@
     <t>Bệnh viện Nhi đồng 1: 532 Lý Thái Tổ, P10</t>
   </si>
   <si>
+    <t>HD023972</t>
+  </si>
+  <si>
+    <t>433/11, Lê Đức Thọ, Phường 17</t>
+  </si>
+  <si>
+    <t>chị hương fb Kim Tien Pham</t>
+  </si>
+  <si>
     <t>HD24001</t>
   </si>
   <si>
@@ -6510,6 +6557,9 @@
     <t>HD024017</t>
   </si>
   <si>
+    <t>190 võ văn ngân</t>
+  </si>
+  <si>
     <t>Cô Kiều Hương fb Vân Trần</t>
   </si>
   <si>
@@ -6528,6 +6578,12 @@
     <t>phạm minh phi_F3: Theer To Lao</t>
   </si>
   <si>
+    <t>HD024093</t>
+  </si>
+  <si>
+    <t>33 đường số 6 p26</t>
+  </si>
+  <si>
     <t>Diễm Phúc</t>
   </si>
   <si>
@@ -6549,64 +6605,421 @@
     <t>HD024164</t>
   </si>
   <si>
+    <t>Toà Aster - Urbun Green (đối diện Vạn Phúc)</t>
+  </si>
+  <si>
     <t>Linh Nga Anna</t>
   </si>
   <si>
-    <t>khả trinh</t>
-  </si>
-  <si>
-    <t>82/17/20đinh tiên hoàng p1</t>
-  </si>
-  <si>
-    <t>chị hương fb Kim Tien Pham</t>
-  </si>
-  <si>
-    <t>HD024093</t>
-  </si>
-  <si>
-    <t>33 đường số 6 p26</t>
-  </si>
-  <si>
-    <t>190 võ văn ngân</t>
-  </si>
-  <si>
-    <t>HD023972</t>
-  </si>
-  <si>
-    <t>433/11, Lê Đức Thọ, Phường 17</t>
-  </si>
-  <si>
-    <t>201 Đường Hoàng Hoa Thám, Phường 13</t>
-  </si>
-  <si>
-    <t>Nguyễn Trinh</t>
-  </si>
-  <si>
-    <t>29/10c trần thái tông</t>
-  </si>
-  <si>
-    <t>Toà Aster - Urbun Green (đối diện Vạn Phúc)</t>
-  </si>
-  <si>
-    <t>91/12 nguyễn thanh tuyền p1</t>
-  </si>
-  <si>
-    <t>240/6A lê thánh tôn phường bến thành</t>
-  </si>
-  <si>
-    <t>Thủy Heri</t>
-  </si>
-  <si>
-    <t>HD024145</t>
-  </si>
-  <si>
-    <t>184/17/35 bãi sậy phường bình tiên</t>
-  </si>
-  <si>
-    <t>137/84D âu dương lân - p2</t>
-  </si>
-  <si>
-    <t>20B Trần Văn Quang, Phường Bảy Hiền</t>
+    <t>NGAY 29-5</t>
+  </si>
+  <si>
+    <t>Cẩm Tiên</t>
+  </si>
+  <si>
+    <t>HD024200</t>
+  </si>
+  <si>
+    <t>Chung cư topaz dragon 2A 457-459 tạ quang bửu - phường 4</t>
+  </si>
+  <si>
+    <t>AT 29-05</t>
+  </si>
+  <si>
+    <t>29-05-2026</t>
+  </si>
+  <si>
+    <t>Chan (inst char importshop) -BN2441</t>
+  </si>
+  <si>
+    <t>HD024246</t>
+  </si>
+  <si>
+    <t>163 Trương Thị Hoa phường Tân Thới Hiệp</t>
+  </si>
+  <si>
+    <t>Uyên</t>
+  </si>
+  <si>
+    <t>HD024442</t>
+  </si>
+  <si>
+    <t>98 Vườn Lài, phường An Phú Đông</t>
+  </si>
+  <si>
+    <t>HD024203</t>
+  </si>
+  <si>
+    <t>Nguyễn Huỳnh Cẩm Tú</t>
+  </si>
+  <si>
+    <t>HD024247</t>
+  </si>
+  <si>
+    <t>78/63 đường số 11, phường thông tây hội</t>
+  </si>
+  <si>
+    <t>Thùy</t>
+  </si>
+  <si>
+    <t>HD024086</t>
+  </si>
+  <si>
+    <t>175 quốc lộ 1k, linh xuân</t>
+  </si>
+  <si>
+    <t>Minh Hồng Nguyễn</t>
+  </si>
+  <si>
+    <t>HD024438</t>
+  </si>
+  <si>
+    <t>Jasmine 1 Hà đô - 118 Đường 3/2, phường 12</t>
+  </si>
+  <si>
+    <t>Tuyen Nguyen</t>
+  </si>
+  <si>
+    <t>HD024412</t>
+  </si>
+  <si>
+    <t>39/44/6 hoàng bật đạt p15</t>
+  </si>
+  <si>
+    <t>Phương Đoan</t>
+  </si>
+  <si>
+    <t>HD024459</t>
+  </si>
+  <si>
+    <t>số 17 đường số 13 bình hưng hòa</t>
+  </si>
+  <si>
+    <t>Út Nhỏ (thu trần ) (Malaysia)</t>
+  </si>
+  <si>
+    <t>HD024433</t>
+  </si>
+  <si>
+    <t>24/5F, Ấp Đông Lân, Xã Bà Điểm</t>
+  </si>
+  <si>
+    <t>Daisy Le</t>
+  </si>
+  <si>
+    <t>HD024416</t>
+  </si>
+  <si>
+    <t>418 Trường Sa, p2</t>
+  </si>
+  <si>
+    <t>Đào thị thanh tâm</t>
+  </si>
+  <si>
+    <t>HD024429</t>
+  </si>
+  <si>
+    <t>320/16 đường ĐHT 02 Phường đông hưng thuận</t>
+  </si>
+  <si>
+    <t>Ngọc Quyên</t>
+  </si>
+  <si>
+    <t>HD024258</t>
+  </si>
+  <si>
+    <t>148a hòa hưng p13</t>
+  </si>
+  <si>
+    <t>HD024304</t>
+  </si>
+  <si>
+    <t>Block d2, chung cư sài gòn riverside (số 4 đào trí phú thuận)</t>
+  </si>
+  <si>
+    <t>HD024270</t>
+  </si>
+  <si>
+    <t>Kim Anh Phạm</t>
+  </si>
+  <si>
+    <t>HD024302</t>
+  </si>
+  <si>
+    <t>16 cư xá bình minh, dương Bá Trạc, phường 1</t>
+  </si>
+  <si>
+    <t>Tạ Ngọc Mai</t>
+  </si>
+  <si>
+    <t>HD024430</t>
+  </si>
+  <si>
+    <t>Sarimi B1, khu chung cư Sala, P. An Lợi Đông</t>
+  </si>
+  <si>
+    <t>Thúy Duy</t>
+  </si>
+  <si>
+    <t>HD024294</t>
+  </si>
+  <si>
+    <t>539,22 hương lộ 3 phường bình hưng hòa</t>
+  </si>
+  <si>
+    <t>Kim Tuyền</t>
+  </si>
+  <si>
+    <t>HD024441</t>
+  </si>
+  <si>
+    <t>451/40 phạm thế hiển phường 3</t>
+  </si>
+  <si>
+    <t>HD024290</t>
+  </si>
+  <si>
+    <t>BN1B2 mini chouchou Fb.</t>
+  </si>
+  <si>
+    <t>HD024453</t>
+  </si>
+  <si>
+    <t>410 Quang Trung f10</t>
+  </si>
+  <si>
+    <t>NGAY 30-5</t>
+  </si>
+  <si>
+    <t>ĐỨC - FB MT MI Ngo</t>
+  </si>
+  <si>
+    <t>HD024678</t>
+  </si>
+  <si>
+    <t>30-05-2026</t>
+  </si>
+  <si>
+    <t>Phạm Thị Thanh Hồng</t>
+  </si>
+  <si>
+    <t>HD024697</t>
+  </si>
+  <si>
+    <t>AT 30-05</t>
+  </si>
+  <si>
+    <t>Ngọc Vũ</t>
+  </si>
+  <si>
+    <t>HD024689</t>
+  </si>
+  <si>
+    <t>42 đương so 6 binh trưng đông</t>
+  </si>
+  <si>
+    <t>Nguyễn Cẩm Tú</t>
+  </si>
+  <si>
+    <t>HD024680</t>
+  </si>
+  <si>
+    <t>Ái Linh</t>
+  </si>
+  <si>
+    <t>HD024455</t>
+  </si>
+  <si>
+    <t>Kiều Nhi</t>
+  </si>
+  <si>
+    <t>HD024623</t>
+  </si>
+  <si>
+    <t>Nguyễn Thu Phương</t>
+  </si>
+  <si>
+    <t>HD024563</t>
+  </si>
+  <si>
+    <t>Sunrise riverside tháp H Đường Nguyễn hữu thọ</t>
+  </si>
+  <si>
+    <t>Hoàng Thu Thủy</t>
+  </si>
+  <si>
+    <t>HD024597</t>
+  </si>
+  <si>
+    <t>583 Nguyễn Thị Thập, phường Bình Thuận</t>
+  </si>
+  <si>
+    <t>HD024510</t>
+  </si>
+  <si>
+    <t>235 QL13 Cũ, HBP</t>
+  </si>
+  <si>
+    <t>HD024702</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Thùy Tiên</t>
+  </si>
+  <si>
+    <t>HD024686</t>
+  </si>
+  <si>
+    <t>Trần Thị Mỹ Duyên</t>
+  </si>
+  <si>
+    <t>HD024528</t>
+  </si>
+  <si>
+    <t>HD024599</t>
+  </si>
+  <si>
+    <t>Chị Bảo Châu</t>
+  </si>
+  <si>
+    <t>HD024669</t>
+  </si>
+  <si>
+    <t>W3370</t>
+  </si>
+  <si>
+    <t>HD024406</t>
+  </si>
+  <si>
+    <t>Ngọc Diệu</t>
+  </si>
+  <si>
+    <t>HD024379</t>
+  </si>
+  <si>
+    <t>HD024538</t>
+  </si>
+  <si>
+    <t>Võ Hằng</t>
+  </si>
+  <si>
+    <t>HD024527</t>
+  </si>
+  <si>
+    <t>HD024666</t>
+  </si>
+  <si>
+    <t>11 đường 18 phường 4</t>
+  </si>
+  <si>
+    <t>BN6352</t>
+  </si>
+  <si>
+    <t>HD024138</t>
+  </si>
+  <si>
+    <t>HD024670</t>
+  </si>
+  <si>
+    <t>Phạm Duyên</t>
+  </si>
+  <si>
+    <t>HD024075</t>
+  </si>
+  <si>
+    <t>HD024454</t>
+  </si>
+  <si>
+    <t>Đặng Trung</t>
+  </si>
+  <si>
+    <t>HD023933</t>
+  </si>
+  <si>
+    <t>HD024607</t>
+  </si>
+  <si>
+    <t>17/2 đường số 10 p bình trưng tây</t>
+  </si>
+  <si>
+    <t>84 song hành phường an phú</t>
+  </si>
+  <si>
+    <t>Ngô Hoàng Ánh</t>
+  </si>
+  <si>
+    <t>320/16 đường ĐHT 02 phường đông hưng thuận</t>
+  </si>
+  <si>
+    <t>4/2b đường số 26 phương an khánh</t>
+  </si>
+  <si>
+    <t>39 an nhơn phường 17</t>
+  </si>
+  <si>
+    <t>An Nguyen - fb Nguyễn Hoàng Thúy An</t>
+  </si>
+  <si>
+    <t>105/48 Nguyễn tư giản f12</t>
+  </si>
+  <si>
+    <t>Số 107, Đường Dương Quảng Hàm phường 7 (tiệm rửa xe)</t>
+  </si>
+  <si>
+    <t>Irire Intara (phòng 505)</t>
+  </si>
+  <si>
+    <t>A25 Hotel - 51-53-55 Cách Mạng Tháng 8, Phường Bến Thành</t>
+  </si>
+  <si>
+    <t>Panhaketya (zalo_thiemuyen)</t>
+  </si>
+  <si>
+    <t>Pham Ngu Lao A67 Nguyen Trai</t>
+  </si>
+  <si>
+    <t>HD024659</t>
+  </si>
+  <si>
+    <t>206 khu phố Mỹ Hào, Hà Huy tập, P. Tân Phong</t>
+  </si>
+  <si>
+    <t>Sky garden 2, cổng đông 3, phường tân phong</t>
+  </si>
+  <si>
+    <t>Hẻm 95, nhà 95/5D, đường 15, phường tân hưng</t>
+  </si>
+  <si>
+    <t>Cty leading star, lô C đường số 3, KCN Đồng An, Bình Hoà</t>
+  </si>
+  <si>
+    <t>tinh</t>
+  </si>
+  <si>
+    <t>hàng tỉnh</t>
+  </si>
+  <si>
+    <t>luu tra</t>
+  </si>
+  <si>
+    <t>Nhân (fb Cam Phu)</t>
+  </si>
+  <si>
+    <t>132 Le van quoi p bình hưng hòa a</t>
+  </si>
+  <si>
+    <t>1/10/2 nguyễn văn yến phường phú thạnh</t>
+  </si>
+  <si>
+    <t>Anh Hải nhận hàng (Thảo Trần)</t>
+  </si>
+  <si>
+    <t>HD024613</t>
+  </si>
+  <si>
+    <t>số 17 đường số 13 phường bình hưng hòa</t>
+  </si>
+  <si>
+    <t>HD024704</t>
   </si>
 </sst>
 </file>
@@ -6701,7 +7114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -6723,6 +7136,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8251,7 +8667,7 @@
         <v>30</v>
       </c>
       <c r="I35" s="6">
-        <f t="shared" ref="I35:I56" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
         <v>30</v>
       </c>
       <c r="J35" s="6" t="s">
@@ -24207,7 +24623,7 @@
         <v>25</v>
       </c>
       <c r="I35" s="3">
-        <f t="shared" ref="I35:I55" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
         <v>700</v>
       </c>
       <c r="J35" s="3" t="s">
@@ -27073,10 +27489,12 @@
   <dimension ref="A1:Q29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
     <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="42.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
     <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -27153,7 +27571,7 @@
         <v>2115</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>2181</v>
+        <v>2116</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>41</v>
@@ -27169,13 +27587,13 @@
         <v>690</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>2116</v>
+        <v>2117</v>
       </c>
       <c r="K3" s="8" t="s">
         <v>24</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="4" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -27183,13 +27601,13 @@
         <v>18</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>2118</v>
+        <v>2119</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>2119</v>
+        <v>2120</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>2182</v>
+        <v>2121</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>102</v>
@@ -27205,13 +27623,13 @@
         <v>1140</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>2116</v>
+        <v>2117</v>
       </c>
       <c r="K4" s="8" t="s">
         <v>24</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="5" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -27219,13 +27637,13 @@
         <v>18</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>2120</v>
+        <v>2122</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>2121</v>
+        <v>2123</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>2176</v>
+        <v>2124</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>102</v>
@@ -27247,7 +27665,7 @@
         <v>24</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -27255,13 +27673,13 @@
         <v>18</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>2164</v>
+        <v>2125</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>2122</v>
+        <v>2126</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>2165</v>
+        <v>2127</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>81</v>
@@ -27283,7 +27701,7 @@
         <v>24</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="7" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -27291,13 +27709,13 @@
         <v>18</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>2123</v>
+        <v>2128</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>2124</v>
+        <v>2129</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>2177</v>
+        <v>2130</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>63</v>
@@ -27319,7 +27737,7 @@
         <v>24</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="8" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -27327,13 +27745,13 @@
         <v>18</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>2125</v>
+        <v>2131</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>2126</v>
+        <v>2132</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>2127</v>
+        <v>2133</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>63</v>
@@ -27355,7 +27773,7 @@
         <v>24</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="9" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -27366,10 +27784,10 @@
         <v>1633</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>2128</v>
+        <v>2134</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>2129</v>
+        <v>2135</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>63</v>
@@ -27391,7 +27809,7 @@
         <v>24</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="10" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -27399,13 +27817,13 @@
         <v>18</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>2178</v>
+        <v>2136</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>2179</v>
+        <v>2137</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>2180</v>
+        <v>2138</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>127</v>
@@ -27421,13 +27839,13 @@
         <v>-25</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>2116</v>
+        <v>2117</v>
       </c>
       <c r="K10" s="8" t="s">
         <v>24</v>
       </c>
       <c r="L10" s="8" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -27435,13 +27853,13 @@
         <v>18</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>2130</v>
+        <v>2139</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>2131</v>
+        <v>2140</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>2172</v>
+        <v>2141</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>102</v>
@@ -27463,7 +27881,7 @@
         <v>24</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="12" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -27471,13 +27889,13 @@
         <v>18</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>2132</v>
+        <v>2142</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>2133</v>
+        <v>2143</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>2134</v>
+        <v>2144</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>77</v>
@@ -27499,7 +27917,7 @@
         <v>24</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
       <c r="M12" s="3" t="s">
         <v>145</v>
@@ -27510,13 +27928,13 @@
         <v>18</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>2135</v>
+        <v>2145</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>2136</v>
+        <v>2146</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>2137</v>
+        <v>2147</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>85</v>
@@ -27532,13 +27950,13 @@
         <v>820</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>2116</v>
+        <v>2117</v>
       </c>
       <c r="K13" s="8" t="s">
         <v>24</v>
       </c>
       <c r="L13" s="8" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="14" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -27549,7 +27967,7 @@
         <v>2085</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>2138</v>
+        <v>2148</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>2087</v>
@@ -27574,7 +27992,7 @@
         <v>24</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="15" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -27582,13 +28000,13 @@
         <v>18</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>2173</v>
+        <v>2149</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>2139</v>
+        <v>2150</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>2174</v>
+        <v>2151</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>102</v>
@@ -27610,7 +28028,7 @@
         <v>24</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="16" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -27621,7 +28039,7 @@
         <v>1930</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>2140</v>
+        <v>2152</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>1932</v>
@@ -27640,13 +28058,13 @@
         <v>820</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>2116</v>
+        <v>2117</v>
       </c>
       <c r="K16" s="8" t="s">
         <v>24</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="17" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -27654,13 +28072,13 @@
         <v>18</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>2141</v>
+        <v>2153</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>2142</v>
+        <v>2154</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>2143</v>
+        <v>2155</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>29</v>
@@ -27682,7 +28100,7 @@
         <v>24</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="18" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -27690,13 +28108,13 @@
         <v>18</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>2144</v>
+        <v>2156</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>2145</v>
+        <v>2157</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>2146</v>
+        <v>2158</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>308</v>
@@ -27718,7 +28136,7 @@
         <v>24</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="19" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -27729,10 +28147,10 @@
         <v>748</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>2170</v>
+        <v>2159</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>2171</v>
+        <v>2160</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>70</v>
@@ -27754,7 +28172,7 @@
         <v>24</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="20" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -27762,10 +28180,10 @@
         <v>18</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>2166</v>
+        <v>2161</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>2147</v>
+        <v>2162</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>242</v>
@@ -27790,7 +28208,7 @@
         <v>24</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="21" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -27798,13 +28216,13 @@
         <v>18</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>2148</v>
+        <v>2163</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>2149</v>
+        <v>2164</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>2169</v>
+        <v>2165</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>77</v>
@@ -27826,7 +28244,7 @@
         <v>24</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="22" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -27834,13 +28252,13 @@
         <v>18</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>2150</v>
+        <v>2166</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>2151</v>
+        <v>2167</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>2152</v>
+        <v>2168</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>355</v>
@@ -27862,7 +28280,7 @@
         <v>24</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="23" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -27873,10 +28291,10 @@
         <v>1163</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>2153</v>
+        <v>2169</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>2154</v>
+        <v>2170</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>63</v>
@@ -27898,7 +28316,7 @@
         <v>24</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="24" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -27906,13 +28324,13 @@
         <v>18</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>2155</v>
+        <v>2171</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>2167</v>
+        <v>2172</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>2168</v>
+        <v>2173</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>81</v>
@@ -27934,7 +28352,7 @@
         <v>24</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="25" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -27942,13 +28360,13 @@
         <v>18</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>2156</v>
+        <v>2174</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>2157</v>
+        <v>2175</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>2158</v>
+        <v>2176</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>41</v>
@@ -27964,13 +28382,13 @@
         <v>820</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>2116</v>
+        <v>2117</v>
       </c>
       <c r="K25" s="8" t="s">
         <v>24</v>
       </c>
       <c r="L25" s="8" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="26" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -27978,13 +28396,13 @@
         <v>18</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>2159</v>
+        <v>2177</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>2160</v>
+        <v>2178</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>2161</v>
+        <v>2179</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>81</v>
@@ -28006,7 +28424,7 @@
         <v>24</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
       <c r="M26" s="3" t="s">
         <v>145</v>
@@ -28020,10 +28438,10 @@
         <v>150</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>2162</v>
+        <v>2180</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>2175</v>
+        <v>2181</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>77</v>
@@ -28045,7 +28463,7 @@
         <v>24</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="28" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -28056,7 +28474,7 @@
         <v>18</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>2163</v>
+        <v>2182</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>2087</v>
@@ -28081,7 +28499,7 @@
         <v>24</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="29" spans="1:17" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -28132,6 +28550,2031 @@
       </c>
       <c r="Q29" s="11">
         <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
+  <dimension ref="A1:P24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="33" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="114.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2183</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>2184</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>2185</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>2186</v>
+      </c>
+      <c r="F3" s="9">
+        <v>8</v>
+      </c>
+      <c r="G3" s="8">
+        <v>920</v>
+      </c>
+      <c r="H3" s="8">
+        <v>30</v>
+      </c>
+      <c r="I3" s="8">
+        <f t="shared" ref="I3:I24" si="0">G3-H3</f>
+        <v>890</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>2189</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>2190</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>2191</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="3">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3">
+        <v>40</v>
+      </c>
+      <c r="I4" s="3">
+        <f t="shared" si="0"/>
+        <v>-40</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>2192</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>2193</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>2194</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="3">
+        <v>910</v>
+      </c>
+      <c r="H5" s="3">
+        <v>30</v>
+      </c>
+      <c r="I5" s="3">
+        <f t="shared" si="0"/>
+        <v>880</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>2195</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="8">
+        <v>1875</v>
+      </c>
+      <c r="H6" s="8">
+        <v>35</v>
+      </c>
+      <c r="I6" s="8">
+        <f t="shared" si="0"/>
+        <v>1840</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>2196</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>2197</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>2198</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G7" s="3">
+        <v>615</v>
+      </c>
+      <c r="H7" s="3">
+        <v>25</v>
+      </c>
+      <c r="I7" s="3">
+        <f t="shared" si="0"/>
+        <v>590</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>2199</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>2200</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>2201</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G8" s="3">
+        <v>1120</v>
+      </c>
+      <c r="H8" s="3">
+        <v>30</v>
+      </c>
+      <c r="I8" s="3">
+        <f t="shared" si="0"/>
+        <v>1090</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>2202</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>2203</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>2204</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="G9" s="6">
+        <v>795</v>
+      </c>
+      <c r="H9" s="6">
+        <v>25</v>
+      </c>
+      <c r="I9" s="6">
+        <f t="shared" si="0"/>
+        <v>770</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>2205</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>2206</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>2207</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G10" s="3">
+        <v>1145</v>
+      </c>
+      <c r="H10" s="3">
+        <v>25</v>
+      </c>
+      <c r="I10" s="3">
+        <f t="shared" si="0"/>
+        <v>1120</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>2208</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>2209</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>2210</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G11" s="8">
+        <v>1770</v>
+      </c>
+      <c r="H11" s="8">
+        <v>30</v>
+      </c>
+      <c r="I11" s="8">
+        <f t="shared" si="0"/>
+        <v>1740</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="8" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>2211</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>2212</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>2213</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>1335</v>
+      </c>
+      <c r="G12" s="8">
+        <v>825</v>
+      </c>
+      <c r="H12" s="8">
+        <v>35</v>
+      </c>
+      <c r="I12" s="8">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="8" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>2214</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>2215</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>2216</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="G13" s="6">
+        <v>850</v>
+      </c>
+      <c r="H13" s="6">
+        <v>20</v>
+      </c>
+      <c r="I13" s="6">
+        <f t="shared" si="0"/>
+        <v>830</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>2217</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>2218</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>2219</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" s="3">
+        <v>720</v>
+      </c>
+      <c r="H14" s="3">
+        <v>30</v>
+      </c>
+      <c r="I14" s="3">
+        <f t="shared" si="0"/>
+        <v>690</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>2220</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>2221</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>2222</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="G15" s="6">
+        <v>0</v>
+      </c>
+      <c r="H15" s="6">
+        <v>25</v>
+      </c>
+      <c r="I15" s="6">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>2224</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="G16" s="8">
+        <v>1690</v>
+      </c>
+      <c r="H16" s="8">
+        <v>30</v>
+      </c>
+      <c r="I16" s="8">
+        <f t="shared" si="0"/>
+        <v>1660</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="8" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>1388</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>2225</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>1390</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G17" s="3">
+        <v>1290</v>
+      </c>
+      <c r="H17" s="3">
+        <v>30</v>
+      </c>
+      <c r="I17" s="3">
+        <f t="shared" si="0"/>
+        <v>1260</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>2226</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>2227</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>2228</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G18" s="8">
+        <v>620</v>
+      </c>
+      <c r="H18" s="8">
+        <v>30</v>
+      </c>
+      <c r="I18" s="8">
+        <f t="shared" si="0"/>
+        <v>590</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="K18" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="8" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>2229</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>2231</v>
+      </c>
+      <c r="F19" s="4">
+        <v>2</v>
+      </c>
+      <c r="G19" s="3">
+        <v>1020</v>
+      </c>
+      <c r="H19" s="3">
+        <v>30</v>
+      </c>
+      <c r="I19" s="3">
+        <f t="shared" si="0"/>
+        <v>990</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>2232</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>2233</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>2234</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" s="8">
+        <v>8559</v>
+      </c>
+      <c r="H20" s="8">
+        <v>65</v>
+      </c>
+      <c r="I20" s="8">
+        <f t="shared" si="0"/>
+        <v>8494</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="8" t="s">
+        <v>2188</v>
+      </c>
+      <c r="M20" s="8" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>2235</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>2236</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>2237</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G21" s="8">
+        <v>2620</v>
+      </c>
+      <c r="H21" s="8">
+        <v>35</v>
+      </c>
+      <c r="I21" s="8">
+        <f t="shared" si="0"/>
+        <v>2585</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>2187</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="8" t="s">
+        <v>2188</v>
+      </c>
+      <c r="M21" s="8" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>2238</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>1195</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="G22" s="6">
+        <v>915</v>
+      </c>
+      <c r="H22" s="6">
+        <v>25</v>
+      </c>
+      <c r="I22" s="6">
+        <f t="shared" si="0"/>
+        <v>890</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>2239</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0</v>
+      </c>
+      <c r="H23" s="3">
+        <v>30</v>
+      </c>
+      <c r="I23" s="3">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>2241</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G24" s="3">
+        <v>4440</v>
+      </c>
+      <c r="H24" s="3">
+        <v>40</v>
+      </c>
+      <c r="I24" s="3">
+        <f t="shared" si="0"/>
+        <v>4400</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
+  <dimension ref="A1:Q31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="35.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="72.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>721</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>2243</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>2244</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>2297</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G3" s="3">
+        <v>1825</v>
+      </c>
+      <c r="H3" s="3">
+        <v>25</v>
+      </c>
+      <c r="I3" s="3">
+        <f t="shared" ref="I3:I31" si="0">G3-H3</f>
+        <v>1800</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>2246</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>2247</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>2308</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G4" s="6">
+        <v>0</v>
+      </c>
+      <c r="H4" s="6">
+        <v>30</v>
+      </c>
+      <c r="I4" s="6">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>2249</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>2250</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>2251</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" s="3">
+        <v>850</v>
+      </c>
+      <c r="H5" s="3">
+        <v>30</v>
+      </c>
+      <c r="I5" s="3">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>2252</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>2253</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>2307</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="G6" s="6">
+        <v>1730</v>
+      </c>
+      <c r="H6" s="6">
+        <v>30</v>
+      </c>
+      <c r="I6" s="6">
+        <f t="shared" si="0"/>
+        <v>1700</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>2254</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>2255</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>2292</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="3">
+        <v>1110</v>
+      </c>
+      <c r="H7" s="3">
+        <v>30</v>
+      </c>
+      <c r="I7" s="3">
+        <f t="shared" si="0"/>
+        <v>1080</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>2301</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>2291</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>2302</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" s="6">
+        <v>0</v>
+      </c>
+      <c r="H8" s="6">
+        <v>25</v>
+      </c>
+      <c r="I8" s="6">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>2256</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>2257</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>2296</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="3">
+        <v>1740</v>
+      </c>
+      <c r="H9" s="3">
+        <v>30</v>
+      </c>
+      <c r="I9" s="3">
+        <f t="shared" si="0"/>
+        <v>1710</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>2258</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>2259</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>2260</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="6">
+        <v>525</v>
+      </c>
+      <c r="H10" s="6">
+        <v>35</v>
+      </c>
+      <c r="I10" s="6">
+        <f t="shared" si="0"/>
+        <v>490</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>2261</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>2262</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>2263</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="G11" s="6">
+        <v>1110</v>
+      </c>
+      <c r="H11" s="6">
+        <v>30</v>
+      </c>
+      <c r="I11" s="6">
+        <f t="shared" si="0"/>
+        <v>1080</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>2294</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>2264</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>2265</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" s="3">
+        <v>520</v>
+      </c>
+      <c r="H12" s="3">
+        <v>30</v>
+      </c>
+      <c r="I12" s="3">
+        <f t="shared" si="0"/>
+        <v>490</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>2303</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>2266</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>2304</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" s="6">
+        <v>0</v>
+      </c>
+      <c r="H13" s="6">
+        <v>25</v>
+      </c>
+      <c r="I13" s="6">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>2267</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>2268</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>2315</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="G14" s="8">
+        <v>845</v>
+      </c>
+      <c r="H14" s="8">
+        <v>25</v>
+      </c>
+      <c r="I14" s="8">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>2248</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="8" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>2269</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>2270</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>2293</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G15" s="3">
+        <v>550</v>
+      </c>
+      <c r="H15" s="3">
+        <v>30</v>
+      </c>
+      <c r="I15" s="3">
+        <f t="shared" si="0"/>
+        <v>520</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>2271</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="G16" s="6">
+        <v>0</v>
+      </c>
+      <c r="H16" s="6">
+        <v>25</v>
+      </c>
+      <c r="I16" s="6">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>2272</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>2273</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>1051</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="G17" s="8">
+        <v>915</v>
+      </c>
+      <c r="H17" s="8">
+        <v>25</v>
+      </c>
+      <c r="I17" s="8">
+        <f t="shared" si="0"/>
+        <v>890</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>2248</v>
+      </c>
+      <c r="K17" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="8" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>2274</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>2087</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G18" s="3">
+        <v>0</v>
+      </c>
+      <c r="H18" s="3">
+        <v>30</v>
+      </c>
+      <c r="I18" s="3">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>2276</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>2277</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>2314</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G19" s="8">
+        <v>1640</v>
+      </c>
+      <c r="H19" s="8">
+        <v>30</v>
+      </c>
+      <c r="I19" s="8">
+        <f t="shared" si="0"/>
+        <v>1610</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>2248</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="8" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>2217</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>2278</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>2295</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G20" s="3">
+        <v>130</v>
+      </c>
+      <c r="H20" s="3">
+        <v>30</v>
+      </c>
+      <c r="I20" s="3">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>2245</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>2279</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>2280</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>2309</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>2310</v>
+      </c>
+      <c r="G21" s="11">
+        <v>570</v>
+      </c>
+      <c r="H21" s="11">
+        <v>0</v>
+      </c>
+      <c r="I21" s="11">
+        <f t="shared" si="0"/>
+        <v>570</v>
+      </c>
+      <c r="J21" s="11" t="s">
+        <v>2312</v>
+      </c>
+      <c r="K21" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="11" t="s">
+        <v>2245</v>
+      </c>
+      <c r="M21" s="21" t="s">
+        <v>2311</v>
+      </c>
+      <c r="N21" s="22" t="s">
+        <v>265</v>
+      </c>
+      <c r="O21" s="22"/>
+      <c r="P21" s="22" t="s">
+        <v>266</v>
+      </c>
+      <c r="Q21" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>2313</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>2281</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>2282</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G22" s="8">
+        <v>0</v>
+      </c>
+      <c r="H22" s="8">
+        <v>30</v>
+      </c>
+      <c r="I22" s="8">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>2248</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="8" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>2283</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>2284</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0</v>
+      </c>
+      <c r="H23" s="3">
+        <v>0</v>
+      </c>
+      <c r="I23" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>2245</v>
+      </c>
+      <c r="M23" s="3" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>1442</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>2319</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>1444</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G24" s="8">
+        <v>0</v>
+      </c>
+      <c r="H24" s="8">
+        <v>30</v>
+      </c>
+      <c r="I24" s="8">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J24" s="8" t="s">
+        <v>2248</v>
+      </c>
+      <c r="K24" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="8" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>1178</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>2305</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>1180</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="G25" s="6">
+        <v>1185</v>
+      </c>
+      <c r="H25" s="6">
+        <v>25</v>
+      </c>
+      <c r="I25" s="6">
+        <f t="shared" si="0"/>
+        <v>1160</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>2283</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>2285</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G26" s="3">
+        <v>0</v>
+      </c>
+      <c r="H26" s="3">
+        <v>40</v>
+      </c>
+      <c r="I26" s="3">
+        <f t="shared" si="0"/>
+        <v>-40</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>2245</v>
+      </c>
+      <c r="M26" s="3" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>2286</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>2287</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>2300</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G27" s="3">
+        <v>775</v>
+      </c>
+      <c r="H27" s="3">
+        <v>25</v>
+      </c>
+      <c r="I27" s="3">
+        <f t="shared" si="0"/>
+        <v>750</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>2298</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>2288</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>2299</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0</v>
+      </c>
+      <c r="H28" s="3">
+        <v>25</v>
+      </c>
+      <c r="I28" s="3">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>2290</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>2306</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="G29" s="6">
+        <v>1600</v>
+      </c>
+      <c r="H29" s="6">
+        <v>30</v>
+      </c>
+      <c r="I29" s="6">
+        <f t="shared" si="0"/>
+        <v>1570</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L29" s="6" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>2316</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>2317</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>2318</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G30" s="8">
+        <v>0</v>
+      </c>
+      <c r="H30" s="8">
+        <v>30</v>
+      </c>
+      <c r="I30" s="8">
+        <f t="shared" ref="I30" si="1">G30-H30</f>
+        <v>-30</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>2248</v>
+      </c>
+      <c r="K30" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L30" s="8" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>1567</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>630</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G31" s="8">
+        <v>0</v>
+      </c>
+      <c r="H31" s="8">
+        <v>30</v>
+      </c>
+      <c r="I31" s="8">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>2248</v>
+      </c>
+      <c r="K31" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L31" s="8" t="s">
+        <v>2245</v>
       </c>
     </row>
   </sheetData>
@@ -29417,7 +31860,7 @@
         <v>30</v>
       </c>
       <c r="I35" s="6">
-        <f t="shared" ref="I35:I55" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
         <v>2090</v>
       </c>
       <c r="J35" s="6" t="s">
@@ -36600,7 +39043,7 @@
         <v>30</v>
       </c>
       <c r="I35" s="8">
-        <f t="shared" ref="I35:I58" si="1">G35-H35</f>
+        <f t="shared" ref="I35:I66" si="1">G35-H35</f>
         <v>-30</v>
       </c>
       <c r="J35" s="8" t="s">

</xml_diff>